<commit_message>
Add password auth and host event setup
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R41d6c7efe6a14582"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="Rb8b71d8a13104a20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R6439d8029f594be8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Ra7c4369df5ae4ba6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R0836b4a1790448cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rcfedcf92ed4d4633"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K12" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K14" headerRowCount="1">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Work_ID"/>
     <x:tableColumn id="2" name="Date_KST"/>
@@ -790,44 +790,114 @@
       </x:c>
     </x:row>
     <x:row r="12" ht="48" hidden="0" customHeight="1">
-      <x:c r="A12" s="22" t="str">
+      <x:c r="A12" s="19" t="str">
         <x:v>GPT-20260625-011</x:v>
       </x:c>
-      <x:c r="B12" s="23" t="str">
+      <x:c r="B12" s="20" t="str">
         <x:v>2026-06-25</x:v>
       </x:c>
-      <x:c r="C12" s="24" t="str">
-        <x:v>Codex-GPT-5</x:v>
-      </x:c>
-      <x:c r="D12" s="24" t="str">
+      <x:c r="C12" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D12" s="21" t="str">
         <x:v>Automated tests</x:v>
       </x:c>
-      <x:c r="E12" s="24" t="str">
+      <x:c r="E12" s="21" t="str">
         <x:v>Committed</x:v>
       </x:c>
-      <x:c r="F12" s="24" t="str">
+      <x:c r="F12" s="21" t="str">
         <x:v>Extracted reservation domain rules into a pure utility module and added Node built-in test coverage for reservation edit capabilities, candidate slot block reasons, and buffer range construction. Added npm test script and a lightweight TS alias loader for tests.</x:v>
       </x:c>
-      <x:c r="G12" s="24" t="str">
+      <x:c r="G12" s="21" t="str">
         <x:v>Needed repeatable coverage for buffer-time conflict checks and reservation-code management rules before deployment work.</x:v>
       </x:c>
-      <x:c r="H12" s="24" t="str">
+      <x:c r="H12" s="21" t="str">
         <x:v>src/lib/reservations/rules.ts; tests/reservation-rules.test.mjs; tests/ts-alias-loader.mjs; package.json; src/app/actions/reservations.ts; src/components/guest/reservation-management-shell.tsx; TODO.md</x:v>
       </x:c>
-      <x:c r="I12" s="24" t="str">
+      <x:c r="I12" s="21" t="str">
         <x:v>npm test, npm run lint, npm run typecheck, npm run build passed.</x:v>
       </x:c>
-      <x:c r="J12" s="24" t="str">
+      <x:c r="J12" s="21" t="str">
         <x:v>No new test dependency was added; tests run through Node 23's built-in test runner and TypeScript stripping.</x:v>
       </x:c>
-      <x:c r="K12" s="24" t="str">
+      <x:c r="K12" s="21" t="str">
         <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="48" hidden="0" customHeight="1">
+      <x:c r="A13" s="19" t="str">
+        <x:v>GPT-20260625-012</x:v>
+      </x:c>
+      <x:c r="B13" s="20" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C13" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D13" s="21" t="str">
+        <x:v>Event creation and password auth</x:v>
+      </x:c>
+      <x:c r="E13" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F13" s="21" t="str">
+        <x:v>Changed web auth from recurring email magic links to email verification plus password sign-up/sign-in. Added drag-based initial availability selection to the Host event creation form and extended createEvent to persist selected AVAILABLE time blocks.</x:v>
+      </x:c>
+      <x:c r="G13" s="21" t="str">
+        <x:v>User wanted password login after initial email verification and wanted graduates to set event dates/times through the same drag calendar interaction used elsewhere.</x:v>
+      </x:c>
+      <x:c r="H13" s="21" t="str">
+        <x:v>src/app/actions/auth.ts; src/components/auth/auth-form.tsx; src/app/auth/page.tsx; src/app/actions/events.ts; src/components/host/event-create-form.tsx; src/lib/validators/action-inputs.ts; TODO.md</x:v>
+      </x:c>
+      <x:c r="I13" s="21" t="str">
+        <x:v>npm run lint, npm run typecheck, npm test, npm run build passed.</x:v>
+      </x:c>
+      <x:c r="J13" s="21" t="str">
+        <x:v>Supabase Email provider should support Confirm email for sign-up; users then log in with email/password. Event creation still uses date/time bounds to render a per-day drag grid.</x:v>
+      </x:c>
+      <x:c r="K13" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="48" hidden="0" customHeight="1">
+      <x:c r="A14" s="22" t="str">
+        <x:v>GPT-20260625-013</x:v>
+      </x:c>
+      <x:c r="B14" s="23" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C14" s="24" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D14" s="24" t="str">
+        <x:v>Host RLS stabilization</x:v>
+      </x:c>
+      <x:c r="E14" s="24" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F14" s="24" t="str">
+        <x:v>Changed Host event creation, Host event loading, buffer updates, and Host time block management to verify the logged-in user server-side and then use the Supabase admin client for DB writes/reads.</x:v>
+      </x:c>
+      <x:c r="G14" s="24" t="str">
+        <x:v>User hit an events insert RLS error locally despite being logged in. The fix avoids brittle Server Action JWT propagation for Host-owned operations while preserving explicit Host ownership checks.</x:v>
+      </x:c>
+      <x:c r="H14" s="24" t="str">
+        <x:v>src/app/actions/events.ts; src/app/actions/time-blocks.ts; src/app/host/events/[eventId]/page.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="str">
+        <x:v>npm run lint, npm run typecheck, npm test, npm run build passed.</x:v>
+      </x:c>
+      <x:c r="J14" s="24" t="str">
+        <x:v>If this reappears, confirm SUPABASE_SERVICE_ROLE_KEY exists locally and restart the dev server so Server Actions reload env/code.</x:v>
+      </x:c>
+      <x:c r="K14" s="24" t="str">
+        <x:v>working tree</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R405846702143480b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f22acfaac4e498d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -976,7 +1046,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R789e1abd0c9e4f21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2cbc24386f74e67"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1026,7 +1096,7 @@
         <x:v>Latest pushed commit</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>f6e649d Add web auth flow</x:v>
+        <x:v>2301f48 Add reservation review and management flows</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1050,7 +1120,7 @@
         <x:v>Auth decision</x:v>
       </x:c>
       <x:c r="B8" s="21" t="str">
-        <x:v>MVP uses email magic link only. SMS/phone deferred due provider cost.</x:v>
+        <x:v>MVP uses email verification plus password login. SMS/phone deferred due provider cost.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1069,12 +1139,12 @@
         <x:v>npm test; npm run lint; npm run typecheck; npm run build</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="24" hidden="0" customHeight="1">
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="21" t="str">
         <x:v>Current uncommitted scope</x:v>
       </x:c>
       <x:c r="B11" s="21" t="str">
-        <x:v>Expected clean after committing email-only auth cleanup, Host approval/buffer flow, reservation management page, reservation rule tests, and this handoff workbook.</x:v>
+        <x:v>Password auth conversion, drag-based initial event availability selection, Host RLS stabilization, and this worklog update.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" hidden="0" customHeight="1">
@@ -1088,7 +1158,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96e22bc2b305476b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3d531666de4f91"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Improve home dashboard and scheduling UX
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Ra7c4369df5ae4ba6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R0836b4a1790448cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rcfedcf92ed4d4633"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R03494035361441d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R96393ec6e42b4f6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R4f80b72f581e4095"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K14" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K15" headerRowCount="1">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Work_ID"/>
     <x:tableColumn id="2" name="Date_KST"/>
@@ -187,7 +187,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CurrentStateTable" displayName="CurrentStateTable" ref="A1:B12" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CurrentStateTable" displayName="CurrentStateTable" ref="A1:B13" headerRowCount="1">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="Item"/>
     <x:tableColumn id="2" name="Value"/>
@@ -838,7 +838,7 @@
         <x:v>Event creation and password auth</x:v>
       </x:c>
       <x:c r="E13" s="21" t="str">
-        <x:v>Uncommitted</x:v>
+        <x:v>Committed</x:v>
       </x:c>
       <x:c r="F13" s="21" t="str">
         <x:v>Changed web auth from recurring email magic links to email verification plus password sign-up/sign-in. Added drag-based initial availability selection to the Host event creation form and extended createEvent to persist selected AVAILABLE time blocks.</x:v>
@@ -856,48 +856,83 @@
         <x:v>Supabase Email provider should support Confirm email for sign-up; users then log in with email/password. Event creation still uses date/time bounds to render a per-day drag grid.</x:v>
       </x:c>
       <x:c r="K13" s="21" t="str">
-        <x:v>working tree</x:v>
+        <x:v>35112f6</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="48" hidden="0" customHeight="1">
-      <x:c r="A14" s="22" t="str">
+      <x:c r="A14" s="19" t="str">
         <x:v>GPT-20260625-013</x:v>
       </x:c>
-      <x:c r="B14" s="23" t="str">
+      <x:c r="B14" s="20" t="str">
         <x:v>2026-06-25</x:v>
       </x:c>
-      <x:c r="C14" s="24" t="str">
-        <x:v>Codex-GPT-5</x:v>
-      </x:c>
-      <x:c r="D14" s="24" t="str">
+      <x:c r="C14" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D14" s="21" t="str">
         <x:v>Host RLS stabilization</x:v>
       </x:c>
-      <x:c r="E14" s="24" t="str">
+      <x:c r="E14" s="21" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F14" s="21" t="str">
+        <x:v>Changed Host event creation, Host event loading, buffer updates, and Host time block management to verify the logged-in user server-side and then use the Supabase admin client for DB writes/reads.</x:v>
+      </x:c>
+      <x:c r="G14" s="21" t="str">
+        <x:v>User hit an events insert RLS error locally despite being logged in. The fix avoids brittle Server Action JWT propagation for Host-owned operations while preserving explicit Host ownership checks.</x:v>
+      </x:c>
+      <x:c r="H14" s="21" t="str">
+        <x:v>src/app/actions/events.ts; src/app/actions/time-blocks.ts; src/app/host/events/[eventId]/page.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I14" s="21" t="str">
+        <x:v>npm run lint, npm run typecheck, npm test, npm run build passed.</x:v>
+      </x:c>
+      <x:c r="J14" s="21" t="str">
+        <x:v>If this reappears, confirm SUPABASE_SERVICE_ROLE_KEY exists locally and restart the dev server so Server Actions reload env/code.</x:v>
+      </x:c>
+      <x:c r="K14" s="21" t="str">
+        <x:v>35112f6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="96" hidden="0" customHeight="1">
+      <x:c r="A15" s="22" t="str">
+        <x:v>GPT-20260625-014</x:v>
+      </x:c>
+      <x:c r="B15" s="23" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C15" s="24" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D15" s="24" t="str">
+        <x:v>Home, auth, calendar UX</x:v>
+      </x:c>
+      <x:c r="E15" s="24" t="str">
         <x:v>Uncommitted</x:v>
       </x:c>
-      <x:c r="F14" s="24" t="str">
-        <x:v>Changed Host event creation, Host event loading, buffer updates, and Host time block management to verify the logged-in user server-side and then use the Supabase admin client for DB writes/reads.</x:v>
-      </x:c>
-      <x:c r="G14" s="24" t="str">
-        <x:v>User hit an events insert RLS error locally despite being logged in. The fix avoids brittle Server Action JWT propagation for Host-owned operations while preserving explicit Host ownership checks.</x:v>
-      </x:c>
-      <x:c r="H14" s="24" t="str">
-        <x:v>src/app/actions/events.ts; src/app/actions/time-blocks.ts; src/app/host/events/[eventId]/page.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
-      </x:c>
-      <x:c r="I14" s="24" t="str">
-        <x:v>npm run lint, npm run typecheck, npm test, npm run build passed.</x:v>
-      </x:c>
-      <x:c r="J14" s="24" t="str">
-        <x:v>If this reappears, confirm SUPABASE_SERVICE_ROLE_KEY exists locally and restart the dev server so Server Actions reload env/code.</x:v>
-      </x:c>
-      <x:c r="K14" s="24" t="str">
+      <x:c r="F15" s="24" t="str">
+        <x:v>Rebuilt the home screen around event code, reservation management code, event creation, and logged-in Host/Guest schedule summaries. Added reservation code entry on event pages, copy/share buttons for event URLs and reservation codes, password reset/update flow, signup password condition checks, default event title handling, 10-minute calendar slots, full-day event creation editing, date-range calendar selection, creator-owned reservation password bypass, and overlap-safe selection/time block updates.</x:v>
+      </x:c>
+      <x:c r="G15" s="24" t="str">
+        <x:v>User preview feedback asked for dashboard-first login, clearer access-code hierarchy, copyable codes, password UX feedback, calendar-first event creation, 10-minute increments, no duplicate/overlapping selections, and creator account reservation management.</x:v>
+      </x:c>
+      <x:c r="H15" s="24" t="str">
+        <x:v>src/app/page.tsx; src/app/actions/dashboard.ts; src/app/actions/auth.ts; src/app/actions/reservations.ts; src/components/auth/*; src/components/guest/*; src/components/host/event-create-form.tsx; src/components/host/host-dashboard-shell.tsx; src/components/calendar/time-selection-grid.tsx; src/lib/time/range-set.ts; tests/range-set.test.mjs</x:v>
+      </x:c>
+      <x:c r="I15" s="24" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build passed. Browser checked /, /auth signup tab, and /host/events/new route on localhost:3000.</x:v>
+      </x:c>
+      <x:c r="J15" s="24" t="str">
+        <x:v>Supabase users do not need Supabase accounts. Linkless signup confirmation requires Supabase email template changes to include OTP tokens and an app-side verifyOtp screen. Per-buffer-slot persistent toggles still need a schema decision.</x:v>
+      </x:c>
+      <x:c r="K15" s="24" t="str">
         <x:v>working tree</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f22acfaac4e498d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0943f3f265854405"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1046,7 +1081,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2cbc24386f74e67"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R396a7fc5c14c494c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1101,64 +1136,72 @@
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="21" t="str">
-        <x:v>Local dev URL</x:v>
+        <x:v>Latest local commit</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>http://localhost:3001</x:v>
+        <x:v>35112f6 Add password auth and host event setup</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="21" t="str">
-        <x:v>Supabase project</x:v>
+        <x:v>Local dev URL</x:v>
       </x:c>
       <x:c r="B7" s="21" t="str">
-        <x:v>fnmxtfzogbmkchacvhse / ap-northeast-1</x:v>
+        <x:v>http://localhost:3000</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="21" t="str">
-        <x:v>Auth decision</x:v>
+        <x:v>Supabase project</x:v>
       </x:c>
       <x:c r="B8" s="21" t="str">
-        <x:v>MVP uses email verification plus password login. SMS/phone deferred due provider cost.</x:v>
+        <x:v>fnmxtfzogbmkchacvhse / ap-northeast-1</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="21" t="str">
-        <x:v>Secrets policy</x:v>
+        <x:v>Auth decision</x:v>
       </x:c>
       <x:c r="B9" s="21" t="str">
-        <x:v>.env.local exists locally and is gitignored. Do not paste secrets into chats or handoff docs.</x:v>
+        <x:v>MVP uses email verification plus password login. SMS/phone deferred due provider cost.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="21" t="str">
-        <x:v>Recent verification</x:v>
+        <x:v>Secrets policy</x:v>
       </x:c>
       <x:c r="B10" s="21" t="str">
-        <x:v>npm test; npm run lint; npm run typecheck; npm run build</x:v>
+        <x:v>.env.local exists locally and is gitignored. Do not paste secrets into chats or handoff docs.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="21" t="str">
+        <x:v>Recent verification</x:v>
+      </x:c>
+      <x:c r="B11" s="21" t="str">
+        <x:v>npm test; npm run lint; npm run typecheck; npm run build</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" hidden="0" customHeight="1">
+      <x:c r="A12" s="21" t="str">
         <x:v>Current uncommitted scope</x:v>
       </x:c>
-      <x:c r="B11" s="21" t="str">
-        <x:v>Password auth conversion, drag-based initial event availability selection, Host RLS stabilization, and this worklog update.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="24" hidden="0" customHeight="1">
-      <x:c r="A12" s="24" t="str">
+      <x:c r="B12" s="21" t="str">
+        <x:v>Home dashboard/access-code hierarchy, copy buttons, password reset/update UX, event creation calendar UX, 10-minute selection, overlap-safe selection utilities, and this worklog update.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="24" hidden="0" customHeight="1">
+      <x:c r="A13" s="24" t="str">
         <x:v>Recommended next work</x:v>
       </x:c>
-      <x:c r="B12" s="24" t="str">
-        <x:v>Configure Vercel/Supabase deploy URLs; broaden tests around Server Action integration once a test database strategy is chosen.</x:v>
+      <x:c r="B13" s="24" t="str">
+        <x:v>Choose schema for per-buffer-slot toggles, decide whether Supabase email templates should switch to OTP code confirmation, then configure Vercel/Supabase deploy URLs.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb3d531666de4f91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85e942ce9f084038"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add magic link auth and scheduling controls
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R03494035361441d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R96393ec6e42b4f6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R4f80b72f581e4095"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R085de4a9404041a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R14dd3499bf2b4673"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rf7656bd851544b30"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K15" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K16" headerRowCount="1">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Work_ID"/>
     <x:tableColumn id="2" name="Date_KST"/>
@@ -895,44 +895,79 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="96" hidden="0" customHeight="1">
-      <x:c r="A15" s="22" t="str">
+      <x:c r="A15" s="19" t="str">
         <x:v>GPT-20260625-014</x:v>
       </x:c>
-      <x:c r="B15" s="23" t="str">
+      <x:c r="B15" s="20" t="str">
         <x:v>2026-06-25</x:v>
       </x:c>
-      <x:c r="C15" s="24" t="str">
-        <x:v>Codex-GPT-5</x:v>
-      </x:c>
-      <x:c r="D15" s="24" t="str">
+      <x:c r="C15" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D15" s="21" t="str">
         <x:v>Home, auth, calendar UX</x:v>
       </x:c>
-      <x:c r="E15" s="24" t="str">
-        <x:v>Uncommitted</x:v>
-      </x:c>
-      <x:c r="F15" s="24" t="str">
+      <x:c r="E15" s="21" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F15" s="21" t="str">
         <x:v>Rebuilt the home screen around event code, reservation management code, event creation, and logged-in Host/Guest schedule summaries. Added reservation code entry on event pages, copy/share buttons for event URLs and reservation codes, password reset/update flow, signup password condition checks, default event title handling, 10-minute calendar slots, full-day event creation editing, date-range calendar selection, creator-owned reservation password bypass, and overlap-safe selection/time block updates.</x:v>
       </x:c>
-      <x:c r="G15" s="24" t="str">
+      <x:c r="G15" s="21" t="str">
         <x:v>User preview feedback asked for dashboard-first login, clearer access-code hierarchy, copyable codes, password UX feedback, calendar-first event creation, 10-minute increments, no duplicate/overlapping selections, and creator account reservation management.</x:v>
       </x:c>
-      <x:c r="H15" s="24" t="str">
+      <x:c r="H15" s="21" t="str">
         <x:v>src/app/page.tsx; src/app/actions/dashboard.ts; src/app/actions/auth.ts; src/app/actions/reservations.ts; src/components/auth/*; src/components/guest/*; src/components/host/event-create-form.tsx; src/components/host/host-dashboard-shell.tsx; src/components/calendar/time-selection-grid.tsx; src/lib/time/range-set.ts; tests/range-set.test.mjs</x:v>
       </x:c>
-      <x:c r="I15" s="24" t="str">
+      <x:c r="I15" s="21" t="str">
         <x:v>npm run typecheck, npm run lint, npm test, npm run build passed. Browser checked /, /auth signup tab, and /host/events/new route on localhost:3000.</x:v>
       </x:c>
-      <x:c r="J15" s="24" t="str">
+      <x:c r="J15" s="21" t="str">
         <x:v>Supabase users do not need Supabase accounts. Linkless signup confirmation requires Supabase email template changes to include OTP tokens and an app-side verifyOtp screen. Per-buffer-slot persistent toggles still need a schema decision.</x:v>
       </x:c>
-      <x:c r="K15" s="24" t="str">
-        <x:v>working tree</x:v>
+      <x:c r="K15" s="21" t="str">
+        <x:v>d0376ca</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="108" hidden="0" customHeight="1">
+      <x:c r="A16" s="22" t="str">
+        <x:v>GPT-20260625-015</x:v>
+      </x:c>
+      <x:c r="B16" s="23" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C16" s="24" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D16" s="24" t="str">
+        <x:v>Magic link and scheduling UX</x:v>
+      </x:c>
+      <x:c r="E16" s="24" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F16" s="24" t="str">
+        <x:v>Reverted web auth to email magic link only, removed password update route/form, added event buffer direction columns plus per-slot buffer override table/action, added Host date-range edit modal, individual buffer on/off controls, group-focused pending visibility, approve-to-pending cancellation, Host-code redirect to admin, richer reservation slot labels/tooltips, stronger hourly grid lines, Guest buffer direction display, and a 7-day home schedule panel.</x:v>
+      </x:c>
+      <x:c r="G16" s="24" t="str">
+        <x:v>User decided to avoid OTP/password SMTP/template complexity for MVP and requested finer Host calendar controls, clearer reservation visibility, and a dashboard calendar that shows Host and Guest schedules immediately after login.</x:v>
+      </x:c>
+      <x:c r="H16" s="24" t="str">
+        <x:v>src/app/actions/auth.ts; src/app/actions/events.ts; src/app/actions/reservations.ts; src/app/actions/time-blocks.ts; src/app/page.tsx; src/app/event/[eventCode]/page.tsx; src/app/host/events/[eventId]/page.tsx; src/components/auth/*; src/components/calendar/time-selection-grid.tsx; src/components/guest/*; src/components/host/*; src/lib/reservations/rules.ts; src/lib/time/ranges.ts; supabase/migrations/20260625090000_event_buffer_direction_flags.sql</x:v>
+      </x:c>
+      <x:c r="I16" s="24" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build passed.</x:v>
+      </x:c>
+      <x:c r="J16" s="24" t="str">
+        <x:v>Apply the new Supabase migration before using per-slot buffer overrides in a real project. Magic links still require Supabase email delivery and allowed redirect URLs, but no custom SMTP template is required for local MVP testing.</x:v>
+      </x:c>
+      <x:c r="K16" s="24" t="str">
+        <x:v>this commit</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0943f3f265854405"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c4260f676194e3a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1081,7 +1116,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R396a7fc5c14c494c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R513422725f1b48ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1128,7 +1163,7 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="21" t="str">
-        <x:v>Latest pushed commit</x:v>
+        <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
         <x:v>2301f48 Add reservation review and management flows</x:v>
@@ -1136,10 +1171,10 @@
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="21" t="str">
-        <x:v>Latest local commit</x:v>
+        <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>35112f6 Add password auth and host event setup</x:v>
+        <x:v>d0376ca Improve home dashboard and scheduling UX</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1163,7 +1198,7 @@
         <x:v>Auth decision</x:v>
       </x:c>
       <x:c r="B9" s="21" t="str">
-        <x:v>MVP uses email verification plus password login. SMS/phone deferred due provider cost.</x:v>
+        <x:v>MVP uses email magic link only. Password/OTP/SMS flows are deferred to avoid SMTP template and SMS provider setup.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1184,10 +1219,10 @@
     </x:row>
     <x:row r="12" ht="24" hidden="0" customHeight="1">
       <x:c r="A12" s="21" t="str">
-        <x:v>Current uncommitted scope</x:v>
+        <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Home dashboard/access-code hierarchy, copy buttons, password reset/update UX, event creation calendar UX, 10-minute selection, overlap-safe selection utilities, and this worklog update.</x:v>
+        <x:v>Magic link auth simplification, Host date/buffer controls, per-slot buffer override schema/actions, group-focused approval visibility, home 7-day schedule, and this worklog update.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -1195,13 +1230,13 @@
         <x:v>Recommended next work</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Choose schema for per-buffer-slot toggles, decide whether Supabase email templates should switch to OTP code confirmation, then configure Vercel/Supabase deploy URLs.</x:v>
+        <x:v>Run/apply the new Supabase migration, smoke-test Host/Guest flows with real Supabase data, then configure Vercel/Supabase deploy URLs.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85e942ce9f084038"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c0fea06a422484d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Restore password auth without OTP
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R085de4a9404041a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R14dd3499bf2b4673"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rf7656bd851544b30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R153ccf1dd8344286"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R8d7927187a3e4926"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R6838b2058e944136"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K16" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K17" headerRowCount="1">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Work_ID"/>
     <x:tableColumn id="2" name="Date_KST"/>
@@ -930,44 +930,79 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="108" hidden="0" customHeight="1">
-      <x:c r="A16" s="22" t="str">
+      <x:c r="A16" s="19" t="str">
         <x:v>GPT-20260625-015</x:v>
       </x:c>
-      <x:c r="B16" s="23" t="str">
+      <x:c r="B16" s="20" t="str">
         <x:v>2026-06-25</x:v>
       </x:c>
-      <x:c r="C16" s="24" t="str">
-        <x:v>Codex-GPT-5</x:v>
-      </x:c>
-      <x:c r="D16" s="24" t="str">
+      <x:c r="C16" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D16" s="21" t="str">
         <x:v>Magic link and scheduling UX</x:v>
       </x:c>
-      <x:c r="E16" s="24" t="str">
-        <x:v>Committed</x:v>
-      </x:c>
-      <x:c r="F16" s="24" t="str">
+      <x:c r="E16" s="21" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F16" s="21" t="str">
         <x:v>Reverted web auth to email magic link only, removed password update route/form, added event buffer direction columns plus per-slot buffer override table/action, added Host date-range edit modal, individual buffer on/off controls, group-focused pending visibility, approve-to-pending cancellation, Host-code redirect to admin, richer reservation slot labels/tooltips, stronger hourly grid lines, Guest buffer direction display, and a 7-day home schedule panel.</x:v>
       </x:c>
-      <x:c r="G16" s="24" t="str">
+      <x:c r="G16" s="21" t="str">
         <x:v>User decided to avoid OTP/password SMTP/template complexity for MVP and requested finer Host calendar controls, clearer reservation visibility, and a dashboard calendar that shows Host and Guest schedules immediately after login.</x:v>
       </x:c>
-      <x:c r="H16" s="24" t="str">
+      <x:c r="H16" s="21" t="str">
         <x:v>src/app/actions/auth.ts; src/app/actions/events.ts; src/app/actions/reservations.ts; src/app/actions/time-blocks.ts; src/app/page.tsx; src/app/event/[eventCode]/page.tsx; src/app/host/events/[eventId]/page.tsx; src/components/auth/*; src/components/calendar/time-selection-grid.tsx; src/components/guest/*; src/components/host/*; src/lib/reservations/rules.ts; src/lib/time/ranges.ts; supabase/migrations/20260625090000_event_buffer_direction_flags.sql</x:v>
       </x:c>
-      <x:c r="I16" s="24" t="str">
+      <x:c r="I16" s="21" t="str">
         <x:v>npm run typecheck, npm run lint, npm test, npm run build passed.</x:v>
       </x:c>
-      <x:c r="J16" s="24" t="str">
+      <x:c r="J16" s="21" t="str">
         <x:v>Apply the new Supabase migration before using per-slot buffer overrides in a real project. Magic links still require Supabase email delivery and allowed redirect URLs, but no custom SMTP template is required for local MVP testing.</x:v>
       </x:c>
-      <x:c r="K16" s="24" t="str">
+      <x:c r="K16" s="21" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="48" hidden="0" customHeight="1">
+      <x:c r="A17" s="22" t="str">
+        <x:v>GPT-20260625-016</x:v>
+      </x:c>
+      <x:c r="B17" s="23" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C17" s="24" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D17" s="24" t="str">
+        <x:v>Password auth correction</x:v>
+      </x:c>
+      <x:c r="E17" s="24" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F17" s="24" t="str">
+        <x:v>Restored email/password sign-up and sign-in, restored password reset/update link flow, kept password condition and confirmation UI, removed magic-link login behavior, and kept OTP code entry out of the web auth flow.</x:v>
+      </x:c>
+      <x:c r="G17" s="24" t="str">
+        <x:v>User clarified that only OTP code login should be removed; password input/login must remain so users do not authenticate by email every time.</x:v>
+      </x:c>
+      <x:c r="H17" s="24" t="str">
+        <x:v>src/app/actions/auth.ts; src/components/auth/auth-form.tsx; src/app/auth/page.tsx; src/app/auth/update-password/page.tsx; src/components/auth/update-password-form.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build passed.</x:v>
+      </x:c>
+      <x:c r="J17" s="24" t="str">
+        <x:v>Final auth shape: sign-up sends Supabase confirmation email, users then log in with email/password; password reset uses Supabase recovery email link. No OTP screen is present.</x:v>
+      </x:c>
+      <x:c r="K17" s="24" t="str">
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c4260f676194e3a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re994eaefe166406e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1116,7 +1151,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R513422725f1b48ed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54a816e472bb4ec2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1198,7 +1233,7 @@
         <x:v>Auth decision</x:v>
       </x:c>
       <x:c r="B9" s="21" t="str">
-        <x:v>MVP uses email magic link only. Password/OTP/SMS flows are deferred to avoid SMTP template and SMS provider setup.</x:v>
+        <x:v>MVP uses email/password login. Sign-up and password reset use Supabase email links. OTP code entry and SMS are deferred.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1217,12 +1252,12 @@
         <x:v>npm test; npm run lint; npm run typecheck; npm run build</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="24" hidden="0" customHeight="1">
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="21" t="str">
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Magic link auth simplification, Host date/buffer controls, per-slot buffer override schema/actions, group-focused approval visibility, home 7-day schedule, and this worklog update.</x:v>
+        <x:v>Restored password auth after clarifying that only OTP should be removed, plus this worklog update.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -1236,7 +1271,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c0fea06a422484d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79c28f0c9c244075"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refine calendar buffer interactions
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R153ccf1dd8344286"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R8d7927187a3e4926"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R6838b2058e944136"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Ra880d82b1fb7432f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="Rd9c5853648174f62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R9f0a89579e054d31"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K17" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K18" headerRowCount="1">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Work_ID"/>
     <x:tableColumn id="2" name="Date_KST"/>
@@ -965,44 +965,79 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="48" hidden="0" customHeight="1">
-      <x:c r="A17" s="22" t="str">
+      <x:c r="A17" s="19" t="str">
         <x:v>GPT-20260625-016</x:v>
       </x:c>
-      <x:c r="B17" s="23" t="str">
+      <x:c r="B17" s="20" t="str">
         <x:v>2026-06-25</x:v>
       </x:c>
-      <x:c r="C17" s="24" t="str">
-        <x:v>Codex-GPT-5</x:v>
-      </x:c>
-      <x:c r="D17" s="24" t="str">
+      <x:c r="C17" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D17" s="21" t="str">
         <x:v>Password auth correction</x:v>
       </x:c>
-      <x:c r="E17" s="24" t="str">
-        <x:v>Committed</x:v>
-      </x:c>
-      <x:c r="F17" s="24" t="str">
+      <x:c r="E17" s="21" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F17" s="21" t="str">
         <x:v>Restored email/password sign-up and sign-in, restored password reset/update link flow, kept password condition and confirmation UI, removed magic-link login behavior, and kept OTP code entry out of the web auth flow.</x:v>
       </x:c>
-      <x:c r="G17" s="24" t="str">
+      <x:c r="G17" s="21" t="str">
         <x:v>User clarified that only OTP code login should be removed; password input/login must remain so users do not authenticate by email every time.</x:v>
       </x:c>
-      <x:c r="H17" s="24" t="str">
+      <x:c r="H17" s="21" t="str">
         <x:v>src/app/actions/auth.ts; src/components/auth/auth-form.tsx; src/app/auth/page.tsx; src/app/auth/update-password/page.tsx; src/components/auth/update-password-form.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
       </x:c>
-      <x:c r="I17" s="24" t="str">
+      <x:c r="I17" s="21" t="str">
         <x:v>npm run typecheck, npm run lint, npm test, npm run build passed.</x:v>
       </x:c>
-      <x:c r="J17" s="24" t="str">
+      <x:c r="J17" s="21" t="str">
         <x:v>Final auth shape: sign-up sends Supabase confirmation email, users then log in with email/password; password reset uses Supabase recovery email link. No OTP screen is present.</x:v>
       </x:c>
-      <x:c r="K17" s="24" t="str">
+      <x:c r="K17" s="21" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="72" hidden="0" customHeight="1">
+      <x:c r="A18" s="22" t="str">
+        <x:v>GPT-20260625-017</x:v>
+      </x:c>
+      <x:c r="B18" s="23" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C18" s="24" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D18" s="24" t="str">
+        <x:v>Calendar interaction UX</x:v>
+      </x:c>
+      <x:c r="E18" s="24" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F18" s="24" t="str">
+        <x:v>Added active-date storage, custom buffer ranges, discontinuous date grids, multi-date drag selection, availability toggle/resizing, hover popovers for pending/confirmed/buffer blocks, per-buffer add/remove/resize controls, confirmed slot resizing, focused pending visibility rules, buffer settings modal, and Guest/reservation buffer override display.</x:v>
+      </x:c>
+      <x:c r="G18" s="24" t="str">
+        <x:v>User specified detailed Host calendar rules for buffer behavior, pending visibility, hover modals, drag semantics, date toggling, and group list collapse behavior.</x:v>
+      </x:c>
+      <x:c r="H18" s="24" t="str">
+        <x:v>supabase/migrations/20260625110000_calendar_interaction_state.sql; src/app/actions/events.ts; src/app/actions/reservations.ts; src/components/calendar/time-selection-grid.tsx; src/components/host/host-dashboard-shell.tsx; src/hooks/use-time-selection.ts; src/store/use-selection-store.ts; src/lib/time/*; tests/range-set.test.mjs</x:v>
+      </x:c>
+      <x:c r="I18" s="24" t="str">
+        <x:v>npx supabase db push, npm run db:types, npm run typecheck, npm run lint, npm test, npm run build passed.</x:v>
+      </x:c>
+      <x:c r="J18" s="24" t="str">
+        <x:v>event_active_dates drives displayed days while events.date_start/date_end remain min/max. BLOCKED is still supported but should move to a personal calendar model later. Confirmed slot resizing can exceed the original pending slot after a warning.</x:v>
+      </x:c>
+      <x:c r="K18" s="24" t="str">
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re994eaefe166406e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R213cbdb0642a428f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1151,7 +1186,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54a816e472bb4ec2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f436812ef624c00"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1201,7 +1236,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>2301f48 Add reservation review and management flows</x:v>
+        <x:v>c847157 Restore password auth without OTP</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1209,7 +1244,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>d0376ca Improve home dashboard and scheduling UX</x:v>
+        <x:v>c847157 Restore password auth without OTP</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1249,15 +1284,15 @@
         <x:v>Recent verification</x:v>
       </x:c>
       <x:c r="B11" s="21" t="str">
-        <x:v>npm test; npm run lint; npm run typecheck; npm run build</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="15" hidden="0" customHeight="1">
+        <x:v>npx supabase db push; npm run db:types; npm run typecheck; npm run lint; npm test; npm run build</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" hidden="0" customHeight="1">
       <x:c r="A12" s="21" t="str">
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Restored password auth after clarifying that only OTP should be removed, plus this worklog update.</x:v>
+        <x:v>Calendar interaction rules: active dates, multi-date drag, availability toggles/resizing, buffer modal and per-buffer controls, confirmed resize, pending visibility focus, and hover/tap detail popovers.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -1265,13 +1300,13 @@
         <x:v>Recommended next work</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Run/apply the new Supabase migration, smoke-test Host/Guest flows with real Supabase data, then configure Vercel/Supabase deploy URLs.</x:v>
+        <x:v>Smoke-test Host/Guest flows against real Supabase data, then decide personal-calendar BLOCKED refactor and configure Vercel/Supabase deploy URLs.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79c28f0c9c244075"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d781562199d4bdf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refine scheduling calendar UX
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Ra880d82b1fb7432f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="Rd9c5853648174f62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R9f0a89579e054d31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R786ed11d9fd14759"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="Raefec36c14484cf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Ra3bacb66861b4845"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K18" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K37" headerRowCount="1">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Work_ID"/>
     <x:tableColumn id="2" name="Date_KST"/>
@@ -1000,44 +1000,709 @@
       </x:c>
     </x:row>
     <x:row r="18" ht="72" hidden="0" customHeight="1">
-      <x:c r="A18" s="22" t="str">
+      <x:c r="A18" s="19" t="str">
         <x:v>GPT-20260625-017</x:v>
       </x:c>
-      <x:c r="B18" s="23" t="str">
-        <x:v>2026-06-25</x:v>
-      </x:c>
-      <x:c r="C18" s="24" t="str">
-        <x:v>Codex-GPT-5</x:v>
-      </x:c>
-      <x:c r="D18" s="24" t="str">
+      <x:c r="B18" s="20" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C18" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D18" s="21" t="str">
         <x:v>Calendar interaction UX</x:v>
       </x:c>
-      <x:c r="E18" s="24" t="str">
+      <x:c r="E18" s="21" t="str">
         <x:v>Committed</x:v>
       </x:c>
-      <x:c r="F18" s="24" t="str">
+      <x:c r="F18" s="21" t="str">
         <x:v>Added active-date storage, custom buffer ranges, discontinuous date grids, multi-date drag selection, availability toggle/resizing, hover popovers for pending/confirmed/buffer blocks, per-buffer add/remove/resize controls, confirmed slot resizing, focused pending visibility rules, buffer settings modal, and Guest/reservation buffer override display.</x:v>
       </x:c>
-      <x:c r="G18" s="24" t="str">
+      <x:c r="G18" s="21" t="str">
         <x:v>User specified detailed Host calendar rules for buffer behavior, pending visibility, hover modals, drag semantics, date toggling, and group list collapse behavior.</x:v>
       </x:c>
-      <x:c r="H18" s="24" t="str">
+      <x:c r="H18" s="21" t="str">
         <x:v>supabase/migrations/20260625110000_calendar_interaction_state.sql; src/app/actions/events.ts; src/app/actions/reservations.ts; src/components/calendar/time-selection-grid.tsx; src/components/host/host-dashboard-shell.tsx; src/hooks/use-time-selection.ts; src/store/use-selection-store.ts; src/lib/time/*; tests/range-set.test.mjs</x:v>
       </x:c>
-      <x:c r="I18" s="24" t="str">
+      <x:c r="I18" s="21" t="str">
         <x:v>npx supabase db push, npm run db:types, npm run typecheck, npm run lint, npm test, npm run build passed.</x:v>
       </x:c>
-      <x:c r="J18" s="24" t="str">
+      <x:c r="J18" s="21" t="str">
         <x:v>event_active_dates drives displayed days while events.date_start/date_end remain min/max. BLOCKED is still supported but should move to a personal calendar model later. Confirmed slot resizing can exceed the original pending slot after a warning.</x:v>
       </x:c>
-      <x:c r="K18" s="24" t="str">
+      <x:c r="K18" s="21" t="str">
         <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="72" hidden="0" customHeight="1">
+      <x:c r="A19" s="19" t="str">
+        <x:v>GPT-20260625-018</x:v>
+      </x:c>
+      <x:c r="B19" s="20" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C19" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D19" s="21" t="str">
+        <x:v>Event creation calendar UX</x:v>
+      </x:c>
+      <x:c r="E19" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F19" s="21" t="str">
+        <x:v>Changed the new-event date picker to active/inactive date toggling with drag preview, added activeDates support to createEvent persistence, hid the new-event selected-count footer, enlarged the new-event 10-minute grid rows, changed the shared time axis to compact AM/PM labels, and made Host availability changes auto-save immediately after drag.</x:v>
+      </x:c>
+      <x:c r="G19" s="21" t="str">
+        <x:v>User wanted the same date deactivation logic on event creation, less visual clutter in the new-event calendar, direct drag-to-save behavior on the management page, and shorter time labels like 8PM instead of Korean full time strings.</x:v>
+      </x:c>
+      <x:c r="H19" s="21" t="str">
+        <x:v>src/components/host/event-create-form.tsx; src/app/actions/events.ts; src/components/calendar/time-selection-grid.tsx; src/components/host/host-dashboard-shell.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I19" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build passed.</x:v>
+      </x:c>
+      <x:c r="J19" s="21" t="str">
+        <x:v>The working tree contains these changes but they are not committed yet. New events now persist only selected active dates into event_active_dates while date_start/date_end remain the min/max active dates.</x:v>
+      </x:c>
+      <x:c r="K19" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="108" hidden="0" customHeight="1">
+      <x:c r="A20" s="19" t="str">
+        <x:v>GPT-20260625-019</x:v>
+      </x:c>
+      <x:c r="B20" s="20" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C20" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D20" s="21" t="str">
+        <x:v>Calendar privacy and priority UX</x:v>
+      </x:c>
+      <x:c r="E20" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F20" s="21" t="str">
+        <x:v>Added confirmed-slot display time overrides so resizing a confirmed appointment does not mutate the original pending candidate, added reservation slot priority_order persistence, anonymized Guest/Public reservation slot display, redirected new reservations directly to the management page, added Guest candidate priority ordering/reordering/date labels/resizing, constrained Host hover popovers, changed buffer add controls to +버퍼 only where no buffer exists, and added direct buffer trash controls.</x:v>
+      </x:c>
+      <x:c r="G20" s="21" t="str">
+        <x:v>User wanted pending and confirmed slot sizes to remain independent, guests to manage preferred candidate order, guests to avoid seeing other groups' details, and Host buffer/hover controls to be usable without leaving the calendar bounds.</x:v>
+      </x:c>
+      <x:c r="H20" s="21" t="str">
+        <x:v>supabase/migrations/20260625123000_confirmed_slot_time_overrides.sql; supabase/migrations/20260625124000_reservation_slot_priority.sql; src/app/actions/reservations.ts; src/app/actions/time-blocks.ts; src/components/calendar/time-selection-grid.tsx; src/components/guest/*; src/components/host/host-dashboard-shell.tsx; src/lib/reservations/slots.ts; src/store/use-selection-store.ts; src/hooks/use-time-selection.ts; tests/range-set.test.mjs</x:v>
+      </x:c>
+      <x:c r="I20" s="21" t="str">
+        <x:v>npx supabase db push, npm run db:types, npm run typecheck, npm run lint, npm test, npm run build passed.</x:v>
+      </x:c>
+      <x:c r="J20" s="21" t="str">
+        <x:v>Superseded by GPT-20260625-020: guests no longer see pending conflicts, even anonymously.</x:v>
+      </x:c>
+      <x:c r="K20" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="108" hidden="0" customHeight="1">
+      <x:c r="A21" s="19" t="str">
+        <x:v>GPT-20260625-020</x:v>
+      </x:c>
+      <x:c r="B21" s="20" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C21" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D21" s="21" t="str">
+        <x:v>Guest privacy and home calendar</x:v>
+      </x:c>
+      <x:c r="E21" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F21" s="21" t="str">
+        <x:v>Changed public Guest/reservation calendars to hide other groups' pending slots entirely, render confirmed slots/buffers/outside-available ranges as generic 불가 blocks, disable waitlist labeling for guests, enlarged the shared 10-minute time grid with a viewport-height minimum, raised the new-event grid row height, and replaced the home '내 7일 일정' panel with a client-side '내 달력' weekly calendar with previous/next week controls, date picker, hover week preview, Sunday-start weeks, today marking, and confirmed-only display for approved reservations.</x:v>
+      </x:c>
+      <x:c r="G21" s="21" t="str">
+        <x:v>User decided guests only need to know possible/impossible availability, not pending competition or buffer details, and wanted the home calendar to behave like a navigable weekly calendar rather than a fixed today-plus-seven list.</x:v>
+      </x:c>
+      <x:c r="H21" s="21" t="str">
+        <x:v>src/components/calendar/time-selection-grid.tsx; src/components/guest/guest-reservation-shell.tsx; src/components/guest/reservation-management-shell.tsx; src/components/home/home-calendar-panel.tsx; src/app/page.tsx; src/lib/time/availability.ts; src/components/host/event-create-form.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I21" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J21" s="21" t="str">
+        <x:v>Superseded by GPT-20260625-021: home calendar is monthly, and guests can select any event-range time while seeing their own candidates.</x:v>
+      </x:c>
+      <x:c r="K21" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="132" hidden="0" customHeight="1">
+      <x:c r="A22" s="19" t="str">
+        <x:v>GPT-20260625-021</x:v>
+      </x:c>
+      <x:c r="B22" s="20" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C22" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D22" s="21" t="str">
+        <x:v>Readable calendar redesign</x:v>
+      </x:c>
+      <x:c r="E22" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F22" s="21" t="str">
+        <x:v>Changed event creation so daily start/end time only controls the visible calendar range and no longer preselects availability, switched visible selection granularity to 30 minutes, changed shared calendar paging to Sunday-Saturday weeks, simplified grid lines to hourly separators, rendered Host drag drafts as actual 가능/불가 blocks instead of '선택 중', centered the buffer trash button inside buffer blocks, removed native title/context tooltips in favor of hover info modals, replaced the home weekly calendar with a monthly dot calendar and hover schedule modal, and allowed approved reservations to keep/show/add pending candidate slots while preserving confirmed slots server-side.</x:v>
+      </x:c>
+      <x:c r="G22" s="21" t="str">
+        <x:v>User wanted large readable calendars, less visual noise, event pages by week, home by month, guests to see their own pending candidates after approval, and candidates to be addable regardless of visible availability.</x:v>
+      </x:c>
+      <x:c r="H22" s="21" t="str">
+        <x:v>src/components/calendar/time-selection-grid.tsx; src/components/host/event-create-form.tsx; src/components/host/host-dashboard-shell.tsx; src/components/guest/guest-reservation-shell.tsx; src/components/guest/reservation-management-shell.tsx; src/components/home/home-calendar-panel.tsx; src/app/actions/reservations.ts; src/lib/reservations/rules.ts; src/app/page.tsx; tests/reservation-rules.test.mjs; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I22" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J22" s="21" t="str">
+        <x:v>Guests no longer see other groups' pending/conflict details, but they can select any visible event-range time. Approved reservations keep confirmed slots and update only unconfirmed candidate slots when saved.</x:v>
+      </x:c>
+      <x:c r="K22" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="84" hidden="0" customHeight="1">
+      <x:c r="A23" s="19" t="str">
+        <x:v>GPT-20260625-022</x:v>
+      </x:c>
+      <x:c r="B23" s="20" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C23" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D23" s="21" t="str">
+        <x:v>Availability drag and date settings</x:v>
+      </x:c>
+      <x:c r="E23" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F23" s="21" t="str">
+        <x:v>Allowed new events to be created without selecting any initial availability, extracted the AM/PM 30-minute time input into a shared calendar component, added daily start/end time editing to the Host date edit modal and Server Action, separated drag commit behavior from drag preview intent, rendered Host availability drag previews by temporarily splitting/toggling visible 가능 blocks, and changed Host draft labels to 가능하게 변경 / 불가능하게 변경.</x:v>
+      </x:c>
+      <x:c r="G23" s="21" t="str">
+        <x:v>User wanted event creation to stop implying that all possible times must be checked up front, wanted date editing to include the default visible time range, and reported that unavailable drag previews were incorrectly labeled as 가능 instead of showing the actual intended change.</x:v>
+      </x:c>
+      <x:c r="H23" s="21" t="str">
+        <x:v>src/components/calendar/meridiem-time-input.tsx; src/components/calendar/time-selection-grid.tsx; src/components/host/event-create-form.tsx; src/components/host/host-dashboard-shell.tsx; src/hooks/use-time-selection.ts; src/store/use-selection-store.ts; src/app/actions/events.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I23" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J23" s="21" t="str">
+        <x:v>Host management still saves availability through the existing toggle Server Action, so preview intent is display-only while commit stays append-style when existing time blocks are present.</x:v>
+      </x:c>
+      <x:c r="K23" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="96" hidden="0" customHeight="1">
+      <x:c r="A24" s="19" t="str">
+        <x:v>GPT-20260625-023</x:v>
+      </x:c>
+      <x:c r="B24" s="20" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C24" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D24" s="21" t="str">
+        <x:v>Panel collapse and priority drag</x:v>
+      </x:c>
+      <x:c r="E24" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F24" s="21" t="str">
+        <x:v>Kept Host availability remove previews visible through autosave so they no longer flash back to 가능 on pointer release, widened the Host date edit modal into a two-column layout, changed collapsed Host reservation groups to show only approval status and participant names, replaced Guest candidate priority arrows with a collapsible drag-handle priority list shared by reservation creation and management, and enlarged the home monthly calendar hover preview.</x:v>
+      </x:c>
+      <x:c r="G24" s="21" t="str">
+        <x:v>User reported a misleading availability flicker, cramped date modal, noisy collapsed group headers, arrow-based priority controls, and tiny home calendar previews.</x:v>
+      </x:c>
+      <x:c r="H24" s="21" t="str">
+        <x:v>src/components/calendar/time-selection-grid.tsx; src/components/host/host-dashboard-shell.tsx; src/components/guest/reservation-priority-list.tsx; src/components/guest/guest-reservation-shell.tsx; src/components/guest/reservation-management-shell.tsx; src/components/home/home-calendar-panel.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I24" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J24" s="21" t="str">
+        <x:v>Priority reordering uses pointer-driven hover target detection instead of native HTML drag so it works more predictably on touch screens.</x:v>
+      </x:c>
+      <x:c r="K24" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="60" hidden="0" customHeight="1">
+      <x:c r="A25" s="19" t="str">
+        <x:v>GPT-20260625-024</x:v>
+      </x:c>
+      <x:c r="B25" s="20" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C25" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D25" s="21" t="str">
+        <x:v>Calendar width and scroll removal</x:v>
+      </x:c>
+      <x:c r="E25" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F25" s="21" t="str">
+        <x:v>Removed the shared time calendar's internal horizontal scroll/min-width, changed calendar columns to fill available parent width, widened CalendarShell and the new-event page to 92rem, and added mobile day paging so narrow viewports show one active date at a time instead of forcing horizontal calendar scroll.</x:v>
+      </x:c>
+      <x:c r="G25" s="21" t="str">
+        <x:v>User wanted calendars to avoid default scrolling and asked to open/spread the layout wide enough for the calendar to be readable without an inner scroll container.</x:v>
+      </x:c>
+      <x:c r="H25" s="21" t="str">
+        <x:v>src/components/calendar/time-selection-grid.tsx; src/components/calendar/calendar-shell.tsx; src/app/host/events/new/page.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I25" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J25" s="21" t="str">
+        <x:v>Desktop calendars show the active week across the full widened page. Mobile calendars page by date to preserve touch targets without horizontal scroll.</x:v>
+      </x:c>
+      <x:c r="K25" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="84" hidden="0" customHeight="1">
+      <x:c r="A26" s="19" t="str">
+        <x:v>GPT-20260625-025</x:v>
+      </x:c>
+      <x:c r="B26" s="20" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C26" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D26" s="21" t="str">
+        <x:v>Home role dashboard and calendar height</x:v>
+      </x:c>
+      <x:c r="E26" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F26" s="21" t="str">
+        <x:v>Increased the shared time calendar slot height/minimum height, compacted the home month calendar height, replaced the stacked home dashboard with a two-column layout that keeps 내 달력 beside a Host/Guest role toggle panel, made Host the default home role with 이벤트 생성 and 내 이벤트, moved 이벤트 코드/예약 관리 코드/내 예약 into the Guest role panel, and added compact code-entry variants for the home panel.</x:v>
+      </x:c>
+      <x:c r="G26" s="21" t="str">
+        <x:v>User clarified that 'no scroll' meant taller event calendars, not only wider calendars, and asked for a simpler home UI that separates Host and Guest roles through toggles instead of a long scrolling stack.</x:v>
+      </x:c>
+      <x:c r="H26" s="21" t="str">
+        <x:v>src/app/page.tsx; src/components/home/home-dashboard-shell.tsx; src/components/home/home-calendar-panel.tsx; src/components/guest/event-code-entry.tsx; src/components/calendar/time-selection-grid.tsx; src/components/host/event-create-form.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I26" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J26" s="21" t="str">
+        <x:v>Home role panels intentionally show the first four events/reservations to keep the first viewport compact; full management remains available through each item's 관리 link.</x:v>
+      </x:c>
+      <x:c r="K26" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="156" hidden="0" customHeight="1">
+      <x:c r="A27" s="19" t="str">
+        <x:v>GPT-20260625-026</x:v>
+      </x:c>
+      <x:c r="B27" s="20" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C27" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D27" s="21" t="str">
+        <x:v>Unified code and calendar polish</x:v>
+      </x:c>
+      <x:c r="E27" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F27" s="21" t="str">
+        <x:v>Added a unified event/reservation access-code resolver and compact code entry, added a Supabase migration that regenerates event and reservation codes until they do not collide across tables, converted the home Host/Guest switch into tab semantics, added 연월 and 오늘 calendar controls, added a shared month-jump modal for event/date pickers, reorganized event creation so title/description stay visible while schedule/buffer and availability are mutually exclusive tabs, widened/reflowed date editing so time controls sit below the calendar, rendered confirmed slots and buffer ranges as generic 불가 blocks on Guest reservation and reservation-management calendars, ensured focused Host pending slots render above confirmed slots, and added copy feedback for link/code buttons.</x:v>
+      </x:c>
+      <x:c r="G27" s="21" t="str">
+        <x:v>User wanted less duplicated access-code UX, guaranteed non-overlapping code routing, clearer calendar navigation, simpler event creation density, Guest visibility of confirmed/buffer unavailability without exposing other pending groups, Host pending overlays above confirmed times, and immediate copy confirmation.</x:v>
+      </x:c>
+      <x:c r="H27" s="21" t="str">
+        <x:v>src/app/actions/access-codes.ts; src/components/guest/access-code-entry.tsx; src/components/home/home-dashboard-shell.tsx; src/components/home/home-calendar-panel.tsx; src/components/calendar/month-jump-dialog.tsx; src/components/calendar/time-selection-grid.tsx; src/components/host/event-create-form.tsx; src/components/host/host-dashboard-shell.tsx; src/components/guest/guest-reservation-shell.tsx; src/components/guest/reservation-management-shell.tsx; src/components/ui/copy-button.tsx; src/lib/reservations/display-ranges.ts; supabase/migrations/20260625133000_distinct_access_codes.sql</x:v>
+      </x:c>
+      <x:c r="I27" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J27" s="21" t="str">
+        <x:v>Run npx supabase db push before relying on cross-table access-code collision protection in the remote database. Guest calendars visually show confirmed/buffer time as unavailable while still allowing candidate selection for waitlist-style requests.</x:v>
+      </x:c>
+      <x:c r="K27" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="108" hidden="0" customHeight="1">
+      <x:c r="A28" s="19" t="str">
+        <x:v>GPT-20260625-027</x:v>
+      </x:c>
+      <x:c r="B28" s="20" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C28" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D28" s="21" t="str">
+        <x:v>Guest availability and reject removal</x:v>
+      </x:c>
+      <x:c r="E28" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F28" s="21" t="str">
+        <x:v>Changed public Guest and reservation-management calendars so confirmed reservations render as 확정 blocks, buffer/confirmed ranges split visible 가능 blocks instead of drawing buffer 불가 overlays, selected candidates show numbered labels such as 후보 1 on the calendar, focused Host pending view also overlays the confirmed slot's original candidate range above the resized confirmed slot, moved +버퍼 controls off the confirmed slot resize edge and raised resize handles, and removed visible reservation rejection buttons from Host slot popovers and group cards.</x:v>
+      </x:c>
+      <x:c r="G28" s="21" t="str">
+        <x:v>User clarified that buffers should divide available time visually rather than appear as unavailable blocks, confirmed reservations must be visible, candidate priority/count must appear on the calendar, focused pending should show over confirmed times, resize edges must remain usable next to buffer controls, and the reject action should not exist in the UI.</x:v>
+      </x:c>
+      <x:c r="H28" s="21" t="str">
+        <x:v>src/lib/time/availability.ts; src/components/calendar/time-selection-grid.tsx; src/components/guest/guest-reservation-shell.tsx; src/components/guest/reservation-management-shell.tsx; src/components/host/host-dashboard-shell.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I28" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J28" s="21" t="str">
+        <x:v>The server-side REJECTED status/action remains for backward compatibility with old data, but no current Host UI exposes a reject button. Public calendars still allow candidate selection even where availability is visually split around confirmed/buffer time.</x:v>
+      </x:c>
+      <x:c r="K28" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="84" hidden="0" customHeight="1">
+      <x:c r="A29" s="19" t="str">
+        <x:v>GPT-20260625-028</x:v>
+      </x:c>
+      <x:c r="B29" s="20" t="str">
+        <x:v>2026-06-25</x:v>
+      </x:c>
+      <x:c r="C29" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D29" s="21" t="str">
+        <x:v>Reservation confirmed display</x:v>
+      </x:c>
+      <x:c r="E29" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F29" s="21" t="str">
+        <x:v>Changed the reservation management calendar so all confirmed slots, including the current reservation group's own confirmed slot, are passed to the public calendar as 확정 blocks. Changed editable selected ranges to include only unconfirmed candidate slots, and allowed approved reservations with an existing confirmed slot to save participant changes even when there are no pending candidate slots.</x:v>
+      </x:c>
+      <x:c r="G29" s="21" t="str">
+        <x:v>User emphasized that confirmed status must be visible on the reservation-holder screen, not only on the public event reservation screen.</x:v>
+      </x:c>
+      <x:c r="H29" s="21" t="str">
+        <x:v>src/components/guest/reservation-management-shell.tsx; src/app/actions/reservations.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I29" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J29" s="21" t="str">
+        <x:v>Approved reservation management now separates 확정 display blocks from editable 후보 selections. Empty requestedSlots are allowed only in the update action so approved reservations can have zero pending candidates while keeping their confirmed slot.</x:v>
+      </x:c>
+      <x:c r="K29" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="168" hidden="0" customHeight="1">
+      <x:c r="A30" s="19" t="str">
+        <x:v>GPT-20260626-029</x:v>
+      </x:c>
+      <x:c r="B30" s="20" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C30" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D30" s="21" t="str">
+        <x:v>Calendar and Host sharing polish</x:v>
+      </x:c>
+      <x:c r="E30" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F30" s="21" t="str">
+        <x:v>Changed the home month label into the 연월 picker button and removed the separate 연월 button, widened the hover bridge for home date previews, added Sunday red and Saturday light-blue tones across home/date/time calendars, changed time-grid date headers to 6/11 (목), removed the separate week-range header row and moved week arrows into the calendar header, added a Host title-adjacent share modal with code/URL copy controls, replaced the old right-panel share block with an active-date-only mini month calendar that controls the visible week, restyled buffer delete/add controls as borderless icon buttons, kept confirmed candidates in reservation-holder right panels while showing 확정(후보 n) on the calendar, and changed Host approval so approving another candidate adds an additional confirmed slot instead of clearing prior confirmed slots.</x:v>
+      </x:c>
+      <x:c r="G30" s="21" t="str">
+        <x:v>User wanted cleaner calendar controls, persistent hover previews, weekend color semantics everywhere, less noisy time-grid headers, sharing near the event title, a mini week navigator in the Host side panel, subtler buffer controls, visible confirmed candidate identity for reservation holders, and additive multi-confirm behavior from the Host right panel.</x:v>
+      </x:c>
+      <x:c r="H30" s="21" t="str">
+        <x:v>src/lib/time/calendar-style.ts; src/components/home/home-calendar-panel.tsx; src/components/calendar/time-selection-grid.tsx; src/components/host/event-create-form.tsx; src/components/host/host-dashboard-shell.tsx; src/components/host/event-share-button.tsx; src/components/calendar/calendar-shell.tsx; src/app/host/events/[eventId]/page.tsx; src/components/guest/reservation-management-shell.tsx; src/components/guest/reservation-priority-list.tsx; src/app/actions/reservations.ts; src/types/domain.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I30" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J30" s="21" t="str">
+        <x:v>Visible Host reject controls remain removed; the legacy REJECTED server status still exists for old data compatibility. Multiple confirmed slots per reservation group are now possible by approving additional pending candidates.</x:v>
+      </x:c>
+      <x:c r="K30" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="132" hidden="0" customHeight="1">
+      <x:c r="A31" s="19" t="str">
+        <x:v>GPT-20260626-030</x:v>
+      </x:c>
+      <x:c r="B31" s="20" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C31" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D31" s="21" t="str">
+        <x:v>Host/home UI refinement</x:v>
+      </x:c>
+      <x:c r="E31" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F31" s="21" t="str">
+        <x:v>Changed the share modal URL copy control to use a link icon, moved Host date editing into a title-adjacent action button and removed the inner 가능 시간 header, moved week navigation into slim first/last day header strips, removed background fills from buffer delete/add icon controls, compacted the Host right-panel reservation groups into bordered collapsible one-line headers, reduced the Host mini calendar height, added dashboard participant loading, showed group names in home calendar previews, changed 내 예약 cards to show status/name/confirmed dated schedules instead of access codes/candidate-only times, and moved Host event codes beside event names.</x:v>
+      </x:c>
+      <x:c r="G31" s="21" t="str">
+        <x:v>User wanted cleaner title-level controls, less noisy Host calendar chrome, clearer collapsible reservation cards, lighter buffer controls, and home panels that identify confirmed groups and useful schedule details without exposing management codes.</x:v>
+      </x:c>
+      <x:c r="H31" s="21" t="str">
+        <x:v>src/components/ui/copy-button.tsx; src/components/host/event-share-button.tsx; src/components/host/event-date-edit-button.tsx; src/app/host/events/[eventId]/page.tsx; src/components/host/host-dashboard-shell.tsx; src/components/calendar/time-selection-grid.tsx; src/app/actions/dashboard.ts; src/components/home/home-calendar-panel.tsx; src/components/home/home-dashboard-shell.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I31" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build passed.</x:v>
+      </x:c>
+      <x:c r="J31" s="21" t="str">
+        <x:v>Expo native apps can reuse shared domain utilities/types and some hooks after platform-neutral extraction, but Next Server Components/Server Actions and DOM/Tailwind UI components cannot be rendered directly in native screens without WebView or platform-specific wrappers.</x:v>
+      </x:c>
+      <x:c r="K31" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="156" hidden="0" customHeight="1">
+      <x:c r="A32" s="19" t="str">
+        <x:v>GPT-20260626-031</x:v>
+      </x:c>
+      <x:c r="B32" s="20" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C32" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D32" s="21" t="str">
+        <x:v>Buffer preview and reservation display fixes</x:v>
+      </x:c>
+      <x:c r="E32" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F32" s="21" t="str">
+        <x:v>Changed Host buffer add controls so hovering the missing before/after half of a confirmed slot renders a translucent buffer time block with a centered plus/spinner, added pending spinners for buffer add/delete, preserved confirmed candidate ranges separately from confirmed display ranges on reservation-management calendars and side panels, rendered adjusted confirmed slots as both a confirmed block and a translucent original-candidate block when their sizes differ, showed guest candidate priority labels to Hosts in calendar labels, popovers, and right-panel rows, changed home 내 예약 rows to show event names instead of participant names, changed date-edit month labels into picker buttons with nested ESC handling, and added optimistic Host time-block state to remove the post-drag save flicker.</x:v>
+      </x:c>
+      <x:c r="G32" s="21" t="str">
+        <x:v>User disliked the floating + buffer button, needed guests and Hosts to see confirmed-vs-candidate size differences correctly, wanted Host visibility into guest priority, wanted home reservation rows keyed by event, and reported a brief revert flicker after availability drag saves.</x:v>
+      </x:c>
+      <x:c r="H32" s="21" t="str">
+        <x:v>src/components/calendar/time-selection-grid.tsx; src/components/guest/reservation-management-shell.tsx; src/components/home/home-dashboard-shell.tsx; src/components/host/event-date-edit-button.tsx; src/components/host/host-dashboard-shell.tsx; src/store/use-selection-store.ts; src/types/domain.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I32" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J32" s="21" t="str">
+        <x:v>Confirmed reservation candidates are now locked out of drag merge/remove operations in the shared selection store; only non-confirmed candidate ranges are editable/saved from reservation management.</x:v>
+      </x:c>
+      <x:c r="K32" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="144" hidden="0" customHeight="1">
+      <x:c r="A33" s="19" t="str">
+        <x:v>GPT-20260626-032</x:v>
+      </x:c>
+      <x:c r="B33" s="20" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C33" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D33" s="21" t="str">
+        <x:v>Calendar interaction corrections</x:v>
+      </x:c>
+      <x:c r="E33" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F33" s="21" t="str">
+        <x:v>Unified the new-event active-date picker with the date-edit picker by making the month label itself open the month jump modal and removing the separate 연월 button, placed month label and 오늘 controls on one row in date-edit, converted time-grid week arrows from header-only buttons into full-height side strips, added Host approval-button hover/focus preview that mutes other pending candidates into a gray patterned tone, moved home calendar status tags beside the group/title line, removed the Host approval restriction that required candidates to be inside AVAILABLE blocks while keeping blocked-time and confirmed/buffer conflict checks, and shifted custom buffer overrides with resized confirmed slots so buffers follow the new confirmed boundaries.</x:v>
+      </x:c>
+      <x:c r="G33" s="21" t="str">
+        <x:v>User clarified the intended month-picker pattern, week-arrow hit area, approval hover preview behavior, approval rules, home modal tag placement, and buffer behavior after confirmed-time resizing.</x:v>
+      </x:c>
+      <x:c r="H33" s="21" t="str">
+        <x:v>src/components/host/event-create-form.tsx; src/components/host/event-date-edit-button.tsx; src/components/calendar/time-selection-grid.tsx; src/components/host/host-dashboard-shell.tsx; src/components/home/home-calendar-panel.tsx; src/app/actions/reservations.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I33" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J33" s="21" t="str">
+        <x:v>Approval now ignores OUTSIDE_AVAILABLE only in Host confirmation/resize validation. Guest candidate creation rules still use the existing availability rule tests.</x:v>
+      </x:c>
+      <x:c r="K33" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="144" hidden="0" customHeight="1">
+      <x:c r="A34" s="19" t="str">
+        <x:v>GPT-20260626-033</x:v>
+      </x:c>
+      <x:c r="B34" s="20" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C34" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D34" s="21" t="str">
+        <x:v>Calendar buffer/debug polish</x:v>
+      </x:c>
+      <x:c r="E34" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F34" s="21" t="str">
+        <x:v>Changed time-grid week navigation from absolute overlays into real grid columns/cells, added reservation-level approval hover focus so confirmed groups can reveal their hidden pending candidates while muting others, made slot popovers measure calendar space and fall back to covering the hovered slot when neither side has room, restyled month labels as button-like month jump controls with underlined 오늘 controls, marked today with circular indicators in event creation/date-edit/week mini calendars, clamped buffer display/resize/save ranges so buffers cannot overlap confirmed slots, and re-anchored active custom buffer overrides when confirmed slots are resized using the event default buffer duration as a maximum.</x:v>
+      </x:c>
+      <x:c r="G34" s="21" t="str">
+        <x:v>User reported approval-hover gaps for already-confirmed groups, shrinking confirmed slots making buffers grow, confusing label-like month controls, missing today circles in mini calendars, week arrows overlaying the table, pending popovers leaving no horizontal room, and buffers/trash icons drifting or overlapping confirmed time.</x:v>
+      </x:c>
+      <x:c r="H34" s="21" t="str">
+        <x:v>src/components/calendar/time-selection-grid.tsx; src/components/host/host-dashboard-shell.tsx; src/components/host/event-create-form.tsx; src/components/host/event-date-edit-button.tsx; src/app/actions/events.ts; src/app/actions/reservations.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I34" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J34" s="21" t="str">
+        <x:v>Buffer overlap prevention now exists in UI preview, Host resize submission, and server-side buffer override saving. Existing malformed buffer overrides are display-clamped and will be corrected when resized/saved or when confirmed slot resize re-anchors active overrides.</x:v>
+      </x:c>
+      <x:c r="K34" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="96" hidden="0" customHeight="1">
+      <x:c r="A35" s="19" t="str">
+        <x:v>GPT-20260626-034</x:v>
+      </x:c>
+      <x:c r="B35" s="20" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C35" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D35" s="21" t="str">
+        <x:v>Home calendar and full-day time UX</x:v>
+      </x:c>
+      <x:c r="E35" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F35" s="21" t="str">
+        <x:v>Changed the home calendar to reuse the shared MonthJumpDialog, centered the month button, moved the underlined 오늘 action to the right controls, made Host slot popovers fall below the slot when no horizontal space exists, disabled rendering of buffer resize handles on the boundary that touches a confirmed slot, added optional label accessories/disabled state to MeridiemTimeInput, and added 0시/자정 preset checkboxes to event creation and date-edit time inputs with end-time 12AM normalized to 24:00.</x:v>
+      </x:c>
+      <x:c r="G35" s="21" t="str">
+        <x:v>User wanted home calendar controls to match the newer month/today pattern, popovers not to cover the hovered slot when side space is unavailable, buffer resize handles not to appear on confirmed-adjacent boundaries, and full-day schedules to be expressible as 00:00 to 24:00 while still enforcing start &lt; end.</x:v>
+      </x:c>
+      <x:c r="H35" s="21" t="str">
+        <x:v>src/components/home/home-calendar-panel.tsx; src/components/calendar/time-selection-grid.tsx; src/components/calendar/meridiem-time-input.tsx; src/components/host/event-create-form.tsx; src/components/host/event-date-edit-button.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I35" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J35" s="21" t="str">
+        <x:v>The UI now treats an end-time 12AM selection as 24:00. Start-time 12AM remains 00:00, so selecting/checking both visible 12AM endpoints represents a full 24-hour day.</x:v>
+      </x:c>
+      <x:c r="K35" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="84" hidden="0" customHeight="1">
+      <x:c r="A36" s="19" t="str">
+        <x:v>GPT-20260626-035</x:v>
+      </x:c>
+      <x:c r="B36" s="20" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C36" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D36" s="21" t="str">
+        <x:v>Calendar hover and today-marker polish</x:v>
+      </x:c>
+      <x:c r="E36" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F36" s="21" t="str">
+        <x:v>Changed Host right-panel cancel buttons to use the same hover/focus preview path as approval buttons while preserving confirmed-slot color with a target ring, changed today indicators in event creation, date-edit, Host week mini calendar, and home month calendar from full circular date cells into small separate markers on normal date buttons/cells, and moved 0시/자정 preset checkboxes directly beside the time input labels.</x:v>
+      </x:c>
+      <x:c r="G36" s="21" t="str">
+        <x:v>User wanted cancel-hover to reveal the affected confirmed slot like approval-hover, disliked today circles replacing the date button shape, and wanted the time preset checkboxes attached immediately next to the labels.</x:v>
+      </x:c>
+      <x:c r="H36" s="21" t="str">
+        <x:v>src/components/calendar/time-selection-grid.tsx; src/components/host/host-dashboard-shell.tsx; src/components/home/home-calendar-panel.tsx; src/components/host/event-create-form.tsx; src/components/host/event-date-edit-button.tsx; src/components/calendar/meridiem-time-input.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I36" s="21" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J36" s="21" t="str">
+        <x:v>Today markers are now visual accents independent from active/selected date button shape. Confirmed cancel hover uses the same preview state as approval hover, so hidden group candidates may temporarily reveal while the confirmed target keeps its primary color.</x:v>
+      </x:c>
+      <x:c r="K36" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="48" hidden="0" customHeight="1">
+      <x:c r="A37" s="22" t="str">
+        <x:v>GPT-20260626-036</x:v>
+      </x:c>
+      <x:c r="B37" s="23" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C37" s="24" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D37" s="24" t="str">
+        <x:v>Final calendar header polish before commit</x:v>
+      </x:c>
+      <x:c r="E37" s="24" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F37" s="24" t="str">
+        <x:v>Moved the event-creation active-date picker 오늘 action to the right-side controls while keeping the month picker centered, and removed the home calendar title row and CalendarDays icon so the month controls lead the panel.</x:v>
+      </x:c>
+      <x:c r="G37" s="24" t="str">
+        <x:v>User wanted the create-event calendar to match the home month-control layout and felt the explicit 내 달력 title/icon looked visually cheap.</x:v>
+      </x:c>
+      <x:c r="H37" s="24" t="str">
+        <x:v>src/components/host/event-create-form.tsx; src/components/home/home-calendar-panel.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I37" s="24" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="J37" s="24" t="str">
+        <x:v>This row was added immediately before committing the accumulated UX batch.</x:v>
+      </x:c>
+      <x:c r="K37" s="24" t="str">
+        <x:v>working tree</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R213cbdb0642a428f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32ede44ea5284fb7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1186,7 +1851,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f436812ef624c00"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55675a4c103b4f70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1220,7 +1885,7 @@
         <x:v>Workspace</x:v>
       </x:c>
       <x:c r="B3" s="21" t="str">
-        <x:v>/Users/0xseo/Desktop/Dev/GradPhotoTime</x:v>
+        <x:v>/Users/0xseo/Documents/GradPhotoTime</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -1236,7 +1901,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>c847157 Restore password auth without OTP</x:v>
+        <x:v>e0077eb Refine calendar buffer interactions</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1244,7 +1909,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>c847157 Restore password auth without OTP</x:v>
+        <x:v>e0077eb Refine calendar buffer interactions</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1284,15 +1949,15 @@
         <x:v>Recent verification</x:v>
       </x:c>
       <x:c r="B11" s="21" t="str">
-        <x:v>npx supabase db push; npm run db:types; npm run typecheck; npm run lint; npm test; npm run build</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="24" hidden="0" customHeight="1">
+        <x:v>npm run typecheck; npm run lint; npm test; npm run build</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="192" hidden="0" customHeight="1">
       <x:c r="A12" s="21" t="str">
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Calendar interaction rules: active dates, multi-date drag, availability toggles/resizing, buffer modal and per-buffer controls, confirmed resize, pending visibility focus, and hover/tap detail popovers.</x:v>
+        <x:v>Uncommitted: event creation visible-range-only availability selection with no required initial availability, shared 30-minute AM/PM time input, new-event and date-edit label-as-month-picker behavior, date modal daily time editing/wider modal with nested ESC behavior, Host drag preview intent labels/split availability preview with optimistic save to avoid release flicker, taller time calendars, no-inner-scroll widened calendars with mobile day paging, simplified home role-toggle dashboard with Host/Guest tabs, unified event/reservation code entry and resolver, cross-table access-code collision trigger migration, compact home month calendar with label-as-picker, reusable month jump modal for small calendars, weekend color semantics across calendars, 6/11 (목) date headers, full-height in-grid time-calendar week arrows, Host title share/date-edit actions, Host mini week navigator, compact collapsible Host group cards with candidate priority and approval-hover candidate muting, translucent hover-directed buffer-add preview blocks with spinners, custom buffers following confirmed-slot resize, Host approval no longer blocked by outside AVAILABLE ranges, collapsible drag-handle Guest priority lists, larger home calendar previews with group names/status tags on one line, 내 예약 confirmed dated schedules by event name without management codes, event codes beside Host event titles, 30-minute readable calendar grid, Sunday-Saturday event paging, monthly home calendar, confirmed-slot display overrides, public Guest availability splitting around confirmed/buffer ranges, numbered candidate labels, reservation-holder 확정 display blocks plus separate adjusted candidate overlays, additive multi-confirm approval, slot priority_order, Guest priority/reorder/resizing, approved-reservation pending candidate editing with locked confirmed candidates, Host pending overlays above confirmed slots, Host buffer/popover usability fixes, and removal of visible Host rejection controls.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -1300,13 +1965,13 @@
         <x:v>Recommended next work</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Smoke-test Host/Guest flows against real Supabase data, then decide personal-calendar BLOCKED refactor and configure Vercel/Supabase deploy URLs.</x:v>
+        <x:v>Commit/push this UX batch after review, run npx supabase db push for the new access-code trigger migration, smoke-test Host/Guest flows against real Supabase data, then configure Vercel/Supabase deploy URLs.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d781562199d4bdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05712b7e35484a2f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Expo mobile shell
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R786ed11d9fd14759"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="Raefec36c14484cf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Ra3bacb66861b4845"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R914354d75c464ec3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R6f74d21e1f7040f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R5591fbce446e4ff7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K37" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K38" headerRowCount="1">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Work_ID"/>
     <x:tableColumn id="2" name="Date_KST"/>
@@ -1665,44 +1665,79 @@
       </x:c>
     </x:row>
     <x:row r="37" ht="48" hidden="0" customHeight="1">
-      <x:c r="A37" s="22" t="str">
+      <x:c r="A37" s="19" t="str">
         <x:v>GPT-20260626-036</x:v>
       </x:c>
-      <x:c r="B37" s="23" t="str">
+      <x:c r="B37" s="20" t="str">
         <x:v>2026-06-26</x:v>
       </x:c>
-      <x:c r="C37" s="24" t="str">
-        <x:v>Codex-GPT-5</x:v>
-      </x:c>
-      <x:c r="D37" s="24" t="str">
+      <x:c r="C37" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D37" s="21" t="str">
         <x:v>Final calendar header polish before commit</x:v>
       </x:c>
-      <x:c r="E37" s="24" t="str">
+      <x:c r="E37" s="21" t="str">
         <x:v>Uncommitted</x:v>
       </x:c>
-      <x:c r="F37" s="24" t="str">
+      <x:c r="F37" s="21" t="str">
         <x:v>Moved the event-creation active-date picker 오늘 action to the right-side controls while keeping the month picker centered, and removed the home calendar title row and CalendarDays icon so the month controls lead the panel.</x:v>
       </x:c>
-      <x:c r="G37" s="24" t="str">
+      <x:c r="G37" s="21" t="str">
         <x:v>User wanted the create-event calendar to match the home month-control layout and felt the explicit 내 달력 title/icon looked visually cheap.</x:v>
       </x:c>
-      <x:c r="H37" s="24" t="str">
+      <x:c r="H37" s="21" t="str">
         <x:v>src/components/host/event-create-form.tsx; src/components/home/home-calendar-panel.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
       </x:c>
-      <x:c r="I37" s="24" t="str">
+      <x:c r="I37" s="21" t="str">
         <x:v>npm run typecheck, npm run lint, npm test, npm run build, git diff --check passed.</x:v>
       </x:c>
-      <x:c r="J37" s="24" t="str">
+      <x:c r="J37" s="21" t="str">
         <x:v>This row was added immediately before committing the accumulated UX batch.</x:v>
       </x:c>
-      <x:c r="K37" s="24" t="str">
+      <x:c r="K37" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="72" hidden="0" customHeight="1">
+      <x:c r="A38" s="22" t="str">
+        <x:v>GPT-20260626-037</x:v>
+      </x:c>
+      <x:c r="B38" s="23" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C38" s="24" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D38" s="24" t="str">
+        <x:v>Expo mobile shell scaffold</x:v>
+      </x:c>
+      <x:c r="E38" s="24" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F38" s="24" t="str">
+        <x:v>Added a `mobile/` Expo WebView shell with native bottom tabs for 내 이벤트, 달력, 참여한 이벤트, and My, plus a floating action button that opens create/join actions by tab context. Added mobile-shell web views for calendar/host/guest home sections, a dedicated `/access` code-entry page, root mobile scripts, mobile ignore rules, and README/TODO setup notes.</x:v>
+      </x:c>
+      <x:c r="G38" s="24" t="str">
+        <x:v>User wanted to start the mobile app with matching functionality/design, a simpler responsive shell, four bottom tabs, and a persistent circular plus button while reusing the existing scheduling flows where possible.</x:v>
+      </x:c>
+      <x:c r="H38" s="24" t="str">
+        <x:v>mobile/App.tsx; mobile/package.json; mobile/app.json; mobile/README.md; mobile/tsconfig.json; src/app/page.tsx; src/app/access/page.tsx; src/components/home/home-dashboard-shell.tsx; package.json; tsconfig.json; README.md; TODO.md; .gitignore; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I38" s="24" t="str">
+        <x:v>npm run typecheck, npm run lint, npm test, npm run build passed. mobile/package.json, app.json, and tsconfig.json parsed successfully. Expo runtime was not executed because mobile dependencies are not installed yet.</x:v>
+      </x:c>
+      <x:c r="J38" s="24" t="str">
+        <x:v>Install mobile dependencies with `cd mobile &amp;&amp; npm install`. Use `EXPO_PUBLIC_WEB_BASE_URL` with a LAN IP for physical-device testing. Future work: configure Universal Links/App Links after production domain and app identifiers are final.</x:v>
+      </x:c>
+      <x:c r="K38" s="24" t="str">
         <x:v>working tree</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32ede44ea5284fb7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92c95ed3909d41f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1851,7 +1886,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55675a4c103b4f70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b836601ef5a47e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1971,7 +2006,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05712b7e35484a2f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81173172bdc642a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add native mobile app API integration
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R914354d75c464ec3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R6f74d21e1f7040f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R5591fbce446e4ff7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Reb1ad1767990460a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R9d6950af52434597"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rd92d8f40eb3a4e16"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K38" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K42" headerRowCount="1">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Work_ID"/>
     <x:tableColumn id="2" name="Date_KST"/>
@@ -1700,44 +1700,184 @@
       </x:c>
     </x:row>
     <x:row r="38" ht="72" hidden="0" customHeight="1">
-      <x:c r="A38" s="22" t="str">
+      <x:c r="A38" s="19" t="str">
         <x:v>GPT-20260626-037</x:v>
       </x:c>
-      <x:c r="B38" s="23" t="str">
+      <x:c r="B38" s="20" t="str">
         <x:v>2026-06-26</x:v>
       </x:c>
-      <x:c r="C38" s="24" t="str">
-        <x:v>Codex-GPT-5</x:v>
-      </x:c>
-      <x:c r="D38" s="24" t="str">
+      <x:c r="C38" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D38" s="21" t="str">
         <x:v>Expo mobile shell scaffold</x:v>
       </x:c>
-      <x:c r="E38" s="24" t="str">
-        <x:v>Uncommitted</x:v>
-      </x:c>
-      <x:c r="F38" s="24" t="str">
+      <x:c r="E38" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F38" s="21" t="str">
         <x:v>Added a `mobile/` Expo WebView shell with native bottom tabs for 내 이벤트, 달력, 참여한 이벤트, and My, plus a floating action button that opens create/join actions by tab context. Added mobile-shell web views for calendar/host/guest home sections, a dedicated `/access` code-entry page, root mobile scripts, mobile ignore rules, and README/TODO setup notes.</x:v>
       </x:c>
-      <x:c r="G38" s="24" t="str">
+      <x:c r="G38" s="21" t="str">
         <x:v>User wanted to start the mobile app with matching functionality/design, a simpler responsive shell, four bottom tabs, and a persistent circular plus button while reusing the existing scheduling flows where possible.</x:v>
       </x:c>
-      <x:c r="H38" s="24" t="str">
+      <x:c r="H38" s="21" t="str">
         <x:v>mobile/App.tsx; mobile/package.json; mobile/app.json; mobile/README.md; mobile/tsconfig.json; src/app/page.tsx; src/app/access/page.tsx; src/components/home/home-dashboard-shell.tsx; package.json; tsconfig.json; README.md; TODO.md; .gitignore; handoff/GradPhotoTime_Worklog.xlsx</x:v>
       </x:c>
-      <x:c r="I38" s="24" t="str">
+      <x:c r="I38" s="21" t="str">
         <x:v>npm run typecheck, npm run lint, npm test, npm run build passed. mobile/package.json, app.json, and tsconfig.json parsed successfully. Expo runtime was not executed because mobile dependencies are not installed yet.</x:v>
       </x:c>
-      <x:c r="J38" s="24" t="str">
+      <x:c r="J38" s="21" t="str">
         <x:v>Install mobile dependencies with `cd mobile &amp;&amp; npm install`. Use `EXPO_PUBLIC_WEB_BASE_URL` with a LAN IP for physical-device testing. Future work: configure Universal Links/App Links after production domain and app identifiers are final.</x:v>
       </x:c>
-      <x:c r="K38" s="24" t="str">
+      <x:c r="K38" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="48" hidden="0" customHeight="1">
+      <x:c r="A39" s="19" t="str">
+        <x:v>GPT-20260626-038</x:v>
+      </x:c>
+      <x:c r="B39" s="20" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C39" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D39" s="21" t="str">
+        <x:v>Expo web runtime dependency fix</x:v>
+      </x:c>
+      <x:c r="E39" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F39" s="21" t="str">
+        <x:v>Added `react-dom` and `react-native-web` to the mobile Expo package and lockfile so Expo web can resolve React Native component exports such as ActivityIndicator.</x:v>
+      </x:c>
+      <x:c r="G39" s="21" t="str">
+        <x:v>User hit `Unable to resolve react-native-web/dist/exports/ActivityIndicator` while running the Expo web bundler; Expo web needs the React DOM and React Native Web runtime packages installed explicitly.</x:v>
+      </x:c>
+      <x:c r="H39" s="21" t="str">
+        <x:v>mobile/package.json; mobile/package-lock.json; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I39" s="21" t="str">
+        <x:v>`npx expo export --platform web --output-dir /private/tmp/gradphoto-mobile-web-export` passed and bundled App.tsx successfully.</x:v>
+      </x:c>
+      <x:c r="J39" s="21" t="str">
+        <x:v>Node 23.11.0 shows React Native engine warnings; use Node 20.19.4, 22.13.0, or 24.3.0+ for a quieter supported toolchain.</x:v>
+      </x:c>
+      <x:c r="K39" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="60" hidden="0" customHeight="1">
+      <x:c r="A40" s="19" t="str">
+        <x:v>GPT-20260626-039</x:v>
+      </x:c>
+      <x:c r="B40" s="20" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C40" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D40" s="21" t="str">
+        <x:v>Mobile deployed-web default URL</x:v>
+      </x:c>
+      <x:c r="E40" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F40" s="21" t="str">
+        <x:v>Changed the Expo mobile WebView default base URL from local Next.js to `https://grad-photo-time.vercel.app` while preserving `EXPO_PUBLIC_WEB_BASE_URL` overrides. Updated mobile and root README instructions so Expo can run against the deployed Vercel app without starting local Next.js.</x:v>
+      </x:c>
+      <x:c r="G40" s="21" t="str">
+        <x:v>User provided the Vercel deployment URL and clarified that mobile testing should not require the local web app when a deployment exists.</x:v>
+      </x:c>
+      <x:c r="H40" s="21" t="str">
+        <x:v>mobile/App.tsx; mobile/README.md; README.md; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I40" s="21" t="str">
+        <x:v>`npx expo export --platform web --output-dir /private/tmp/gradphoto-mobile-web-export-vercel-default` passed. `npm run typecheck` passed.</x:v>
+      </x:c>
+      <x:c r="J40" s="21" t="str">
+        <x:v>Restart Expo with cache clear after this change so the old localhost bundle is not reused.</x:v>
+      </x:c>
+      <x:c r="K40" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="72" hidden="0" customHeight="1">
+      <x:c r="A41" s="19" t="str">
+        <x:v>GPT-20260626-040</x:v>
+      </x:c>
+      <x:c r="B41" s="20" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C41" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D41" s="21" t="str">
+        <x:v>Native Expo mobile UI rewrite</x:v>
+      </x:c>
+      <x:c r="E41" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F41" s="21" t="str">
+        <x:v>Replaced the mobile WebView shell with native React Native screens for the month calendar, Host event list, joined reservation list, My page, event creation form, and unified code entry. Added Expo root registration through `mobile/index.ts`, SDK-compatible package versions, safe-area-context usage, local Android/iOS scripts, and removed WebView/web runtime dependencies.</x:v>
+      </x:c>
+      <x:c r="G41" s="21" t="str">
+        <x:v>User decided the WebView approach made the mobile UI/buttons visually broken and asked for a native rewrite based on the existing product behavior and design direction.</x:v>
+      </x:c>
+      <x:c r="H41" s="21" t="str">
+        <x:v>mobile/App.tsx; mobile/index.ts; mobile/package.json; mobile/package-lock.json; mobile/README.md; README.md; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I41" s="21" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit` passed. `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-native-export` passed. Root `npm run typecheck` passed. `cd mobile &amp;&amp; npx expo install --check` passed.</x:v>
+      </x:c>
+      <x:c r="J41" s="21" t="str">
+        <x:v>Mobile data is currently demo-backed. Next step is to add a mobile API layer through Next.js API routes or Supabase client helpers; do not reintroduce WebView for core screens unless explicitly requested.</x:v>
+      </x:c>
+      <x:c r="K41" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="108" hidden="0" customHeight="1">
+      <x:c r="A42" s="22" t="str">
+        <x:v>GPT-20260626-041</x:v>
+      </x:c>
+      <x:c r="B42" s="23" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C42" s="24" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D42" s="24" t="str">
+        <x:v>Mobile API integration</x:v>
+      </x:c>
+      <x:c r="E42" s="24" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F42" s="24" t="str">
+        <x:v>Added Next.js mobile API routes for email/password sign-in, authenticated dashboard loading, unified event/reservation code resolution, event preview loading, reservation management preview loading, and mobile reservation creation. Connected the native Expo app to those APIs for My tab login, month calendar markers, upcoming schedules, Host event summaries, joined reservation summaries, and code lookup previews with loading/error states.</x:v>
+      </x:c>
+      <x:c r="G42" s="24" t="str">
+        <x:v>The native mobile rewrite needed real Supabase-backed data instead of demo-only screens so device testing can validate actual login, dashboard, and access-code flows while keeping the UI fully native.</x:v>
+      </x:c>
+      <x:c r="H42" s="24" t="str">
+        <x:v>mobile/App.tsx; src/lib/mobile/api-response.ts; src/lib/mobile/auth.ts; src/lib/mobile/dashboard.ts; src/app/api/mobile/auth/sign-in/route.ts; src/app/api/mobile/dashboard/route.ts; src/app/api/mobile/access/resolve/route.ts; src/app/api/mobile/events/[eventCode]/route.ts; src/app/api/mobile/reservations/[accessCode]/route.ts; src/app/api/mobile/reservations/route.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I42" s="24" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-api-export-final` passed. `cd mobile &amp;&amp; npx expo install --check` reported dependencies up to date using the local offline dependency map.</x:v>
+      </x:c>
+      <x:c r="J42" s="24" t="str">
+        <x:v>Mobile event creation and reservation editing screens are still UI scaffolds; the API foundation is ready for wiring native create/reserve/update interactions next. API default base URL is `https://grad-photo-time.vercel.app` unless `EXPO_PUBLIC_API_BASE_URL` is set.</x:v>
+      </x:c>
+      <x:c r="K42" s="24" t="str">
         <x:v>working tree</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92c95ed3909d41f9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb34f9d0193914549"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1886,7 +2026,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b836601ef5a47e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda6778ac60804b9b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2006,7 +2146,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81173172bdc642a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01b83bbaf40d4672"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add mobile refresh creation and session persistence
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Reb1ad1767990460a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R9d6950af52434597"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rd92d8f40eb3a4e16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R56df39411e384138"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R87c7579bf6834af5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R5d7d3b6d8ea04a71"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K42" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K44" headerRowCount="1">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Work_ID"/>
     <x:tableColumn id="2" name="Date_KST"/>
@@ -1840,44 +1840,114 @@
       </x:c>
     </x:row>
     <x:row r="42" ht="108" hidden="0" customHeight="1">
-      <x:c r="A42" s="22" t="str">
+      <x:c r="A42" s="19" t="str">
         <x:v>GPT-20260626-041</x:v>
       </x:c>
-      <x:c r="B42" s="23" t="str">
+      <x:c r="B42" s="20" t="str">
         <x:v>2026-06-26</x:v>
       </x:c>
-      <x:c r="C42" s="24" t="str">
-        <x:v>Codex-GPT-5</x:v>
-      </x:c>
-      <x:c r="D42" s="24" t="str">
+      <x:c r="C42" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D42" s="21" t="str">
         <x:v>Mobile API integration</x:v>
       </x:c>
-      <x:c r="E42" s="24" t="str">
-        <x:v>Uncommitted</x:v>
-      </x:c>
-      <x:c r="F42" s="24" t="str">
+      <x:c r="E42" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F42" s="21" t="str">
         <x:v>Added Next.js mobile API routes for email/password sign-in, authenticated dashboard loading, unified event/reservation code resolution, event preview loading, reservation management preview loading, and mobile reservation creation. Connected the native Expo app to those APIs for My tab login, month calendar markers, upcoming schedules, Host event summaries, joined reservation summaries, and code lookup previews with loading/error states.</x:v>
       </x:c>
-      <x:c r="G42" s="24" t="str">
+      <x:c r="G42" s="21" t="str">
         <x:v>The native mobile rewrite needed real Supabase-backed data instead of demo-only screens so device testing can validate actual login, dashboard, and access-code flows while keeping the UI fully native.</x:v>
       </x:c>
-      <x:c r="H42" s="24" t="str">
+      <x:c r="H42" s="21" t="str">
         <x:v>mobile/App.tsx; src/lib/mobile/api-response.ts; src/lib/mobile/auth.ts; src/lib/mobile/dashboard.ts; src/app/api/mobile/auth/sign-in/route.ts; src/app/api/mobile/dashboard/route.ts; src/app/api/mobile/access/resolve/route.ts; src/app/api/mobile/events/[eventCode]/route.ts; src/app/api/mobile/reservations/[accessCode]/route.ts; src/app/api/mobile/reservations/route.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
       </x:c>
-      <x:c r="I42" s="24" t="str">
+      <x:c r="I42" s="21" t="str">
         <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-api-export-final` passed. `cd mobile &amp;&amp; npx expo install --check` reported dependencies up to date using the local offline dependency map.</x:v>
       </x:c>
-      <x:c r="J42" s="24" t="str">
+      <x:c r="J42" s="21" t="str">
         <x:v>Mobile event creation and reservation editing screens are still UI scaffolds; the API foundation is ready for wiring native create/reserve/update interactions next. API default base URL is `https://grad-photo-time.vercel.app` unless `EXPO_PUBLIC_API_BASE_URL` is set.</x:v>
       </x:c>
-      <x:c r="K42" s="24" t="str">
+      <x:c r="K42" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="72" hidden="0" customHeight="1">
+      <x:c r="A43" s="19" t="str">
+        <x:v>GPT-20260626-042</x:v>
+      </x:c>
+      <x:c r="B43" s="20" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C43" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D43" s="21" t="str">
+        <x:v>Mobile refresh and event creation</x:v>
+      </x:c>
+      <x:c r="E43" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F43" s="21" t="str">
+        <x:v>Added mobile month-calendar date tapping so days with schedules open an inline schedule preview, while empty days only select the date. Added pull-to-refresh on authenticated dashboard tabs. Added a Bearer-token mobile event creation API and wired the native event creation form to create real events, refresh the dashboard, and return to the Host events tab.</x:v>
+      </x:c>
+      <x:c r="G43" s="21" t="str">
+        <x:v>User confirmed the native app works and asked for date-tap schedule visibility, refresh, and actual event creation/other feature wiring for mobile testing.</x:v>
+      </x:c>
+      <x:c r="H43" s="21" t="str">
+        <x:v>mobile/App.tsx; src/app/api/mobile/events/route.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I43" s="21" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-refresh-create-export` passed.</x:v>
+      </x:c>
+      <x:c r="J43" s="21" t="str">
+        <x:v>Mobile event creation currently creates the event shell with active dates, daily time range, and buffer settings; native availability drag editing and full Host event management are still next-step work.</x:v>
+      </x:c>
+      <x:c r="K43" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="72" hidden="0" customHeight="1">
+      <x:c r="A44" s="22" t="str">
+        <x:v>GPT-20260626-043</x:v>
+      </x:c>
+      <x:c r="B44" s="23" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C44" s="24" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D44" s="24" t="str">
+        <x:v>Mobile secure session persistence</x:v>
+      </x:c>
+      <x:c r="E44" s="24" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F44" s="24" t="str">
+        <x:v>Installed `expo-secure-store`, added a mobile auth refresh API, persisted mobile sessions locally after login, restored saved sessions on app launch, refreshed near-expired access tokens with refresh tokens, cleared expired saved sessions, and added a My-tab logout action.</x:v>
+      </x:c>
+      <x:c r="G44" s="24" t="str">
+        <x:v>User wanted automatic login via locally saved tokens and asked to remove the visible refresh button in favor of pull-to-refresh.</x:v>
+      </x:c>
+      <x:c r="H44" s="24" t="str">
+        <x:v>mobile/App.tsx; mobile/package.json; mobile/package-lock.json; src/lib/mobile/auth.ts; src/app/api/mobile/auth/refresh/route.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I44" s="24" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-secure-session-export` passed.</x:v>
+      </x:c>
+      <x:c r="J44" s="24" t="str">
+        <x:v>SecureStore is used instead of AsyncStorage because Supabase access/refresh tokens are sensitive. Pull-to-refresh remains available on authenticated tabs; there is no header refresh button.</x:v>
+      </x:c>
+      <x:c r="K44" s="24" t="str">
         <x:v>working tree</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb34f9d0193914549"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3f7e86797574006"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2026,7 +2096,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda6778ac60804b9b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2d24133ce3a4689"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2146,7 +2216,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01b83bbaf40d4672"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cdeb24ac1ba4349"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add mobile event management screen
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R56df39411e384138"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R87c7579bf6834af5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R5d7d3b6d8ea04a71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R222bc67ebda0443a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="Rfe901b6a885f47d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R3c4f32dc925d467c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K44" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K45" headerRowCount="1">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Work_ID"/>
     <x:tableColumn id="2" name="Date_KST"/>
@@ -1910,44 +1910,79 @@
       </x:c>
     </x:row>
     <x:row r="44" ht="72" hidden="0" customHeight="1">
-      <x:c r="A44" s="22" t="str">
+      <x:c r="A44" s="19" t="str">
         <x:v>GPT-20260626-043</x:v>
       </x:c>
-      <x:c r="B44" s="23" t="str">
+      <x:c r="B44" s="20" t="str">
         <x:v>2026-06-26</x:v>
       </x:c>
-      <x:c r="C44" s="24" t="str">
-        <x:v>Codex-GPT-5</x:v>
-      </x:c>
-      <x:c r="D44" s="24" t="str">
+      <x:c r="C44" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D44" s="21" t="str">
         <x:v>Mobile secure session persistence</x:v>
       </x:c>
-      <x:c r="E44" s="24" t="str">
-        <x:v>Uncommitted</x:v>
-      </x:c>
-      <x:c r="F44" s="24" t="str">
+      <x:c r="E44" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F44" s="21" t="str">
         <x:v>Installed `expo-secure-store`, added a mobile auth refresh API, persisted mobile sessions locally after login, restored saved sessions on app launch, refreshed near-expired access tokens with refresh tokens, cleared expired saved sessions, and added a My-tab logout action.</x:v>
       </x:c>
-      <x:c r="G44" s="24" t="str">
+      <x:c r="G44" s="21" t="str">
         <x:v>User wanted automatic login via locally saved tokens and asked to remove the visible refresh button in favor of pull-to-refresh.</x:v>
       </x:c>
-      <x:c r="H44" s="24" t="str">
+      <x:c r="H44" s="21" t="str">
         <x:v>mobile/App.tsx; mobile/package.json; mobile/package-lock.json; src/lib/mobile/auth.ts; src/app/api/mobile/auth/refresh/route.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
       </x:c>
-      <x:c r="I44" s="24" t="str">
+      <x:c r="I44" s="21" t="str">
         <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-secure-session-export` passed.</x:v>
       </x:c>
-      <x:c r="J44" s="24" t="str">
+      <x:c r="J44" s="21" t="str">
         <x:v>SecureStore is used instead of AsyncStorage because Supabase access/refresh tokens are sensitive. Pull-to-refresh remains available on authenticated tabs; there is no header refresh button.</x:v>
       </x:c>
-      <x:c r="K44" s="24" t="str">
+      <x:c r="K44" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="84" hidden="0" customHeight="1">
+      <x:c r="A45" s="22" t="str">
+        <x:v>GPT-20260626-044</x:v>
+      </x:c>
+      <x:c r="B45" s="23" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C45" s="24" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D45" s="24" t="str">
+        <x:v>Mobile event management entry</x:v>
+      </x:c>
+      <x:c r="E45" s="24" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F45" s="24" t="str">
+        <x:v>Added a native mobile event-management route. Host event cards now open a management screen with event code, date range, daily time range, buffer summary, confirmed schedule list, pending candidate list, participant names, candidate priority labels, empty states, and pull-to-refresh. Expanded the mobile dashboard event payload to include daily time and buffer settings needed by the management screen.</x:v>
+      </x:c>
+      <x:c r="G45" s="24" t="str">
+        <x:v>User asked to start the mobile event management page after confirming mobile login/dashboard flows worked.</x:v>
+      </x:c>
+      <x:c r="H45" s="24" t="str">
+        <x:v>mobile/App.tsx; src/lib/mobile/dashboard.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I45" s="24" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, `git diff --check`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-event-manage-export` passed.</x:v>
+      </x:c>
+      <x:c r="J45" s="24" t="str">
+        <x:v>This is the first native management page: read/navigation is wired. Approval/cancel buttons, buffer editing, and availability drag editing are still next-step mobile work.</x:v>
+      </x:c>
+      <x:c r="K45" s="24" t="str">
         <x:v>working tree</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3f7e86797574006"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R378a596785ff4164"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2096,7 +2131,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2d24133ce3a4689"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10a7f3f85e184636"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cdeb24ac1ba4349"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b9b9609dcc844cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Improve mobile auth persistence and review actions
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R222bc67ebda0443a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="Rfe901b6a885f47d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R3c4f32dc925d467c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R3b99ca6561cb4339"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R8512d83dfe094a4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rd15b8e613db04780"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K45" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K46" headerRowCount="1">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Work_ID"/>
     <x:tableColumn id="2" name="Date_KST"/>
@@ -1945,44 +1945,79 @@
       </x:c>
     </x:row>
     <x:row r="45" ht="84" hidden="0" customHeight="1">
-      <x:c r="A45" s="22" t="str">
+      <x:c r="A45" s="19" t="str">
         <x:v>GPT-20260626-044</x:v>
       </x:c>
-      <x:c r="B45" s="23" t="str">
+      <x:c r="B45" s="20" t="str">
         <x:v>2026-06-26</x:v>
       </x:c>
-      <x:c r="C45" s="24" t="str">
-        <x:v>Codex-GPT-5</x:v>
-      </x:c>
-      <x:c r="D45" s="24" t="str">
+      <x:c r="C45" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D45" s="21" t="str">
         <x:v>Mobile event management entry</x:v>
       </x:c>
-      <x:c r="E45" s="24" t="str">
-        <x:v>Uncommitted</x:v>
-      </x:c>
-      <x:c r="F45" s="24" t="str">
+      <x:c r="E45" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F45" s="21" t="str">
         <x:v>Added a native mobile event-management route. Host event cards now open a management screen with event code, date range, daily time range, buffer summary, confirmed schedule list, pending candidate list, participant names, candidate priority labels, empty states, and pull-to-refresh. Expanded the mobile dashboard event payload to include daily time and buffer settings needed by the management screen.</x:v>
       </x:c>
-      <x:c r="G45" s="24" t="str">
+      <x:c r="G45" s="21" t="str">
         <x:v>User asked to start the mobile event management page after confirming mobile login/dashboard flows worked.</x:v>
       </x:c>
-      <x:c r="H45" s="24" t="str">
+      <x:c r="H45" s="21" t="str">
         <x:v>mobile/App.tsx; src/lib/mobile/dashboard.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
       </x:c>
-      <x:c r="I45" s="24" t="str">
+      <x:c r="I45" s="21" t="str">
         <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, `git diff --check`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-event-manage-export` passed.</x:v>
       </x:c>
-      <x:c r="J45" s="24" t="str">
+      <x:c r="J45" s="21" t="str">
         <x:v>This is the first native management page: read/navigation is wired. Approval/cancel buttons, buffer editing, and availability drag editing are still next-step mobile work.</x:v>
       </x:c>
-      <x:c r="K45" s="24" t="str">
+      <x:c r="K45" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="84" hidden="0" customHeight="1">
+      <x:c r="A46" s="22" t="str">
+        <x:v>GPT-20260626-045</x:v>
+      </x:c>
+      <x:c r="B46" s="23" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C46" s="24" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D46" s="24" t="str">
+        <x:v>Mobile auth resilience and review actions</x:v>
+      </x:c>
+      <x:c r="E46" s="24" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F46" s="24" t="str">
+        <x:v>Hardened native mobile session persistence so dashboard refresh failures no longer clear saved sessions unless the API returns 401, added automatic refresh-token retry for dashboard loads, event creation, code lookup, and review actions, added native email/password sign-up UI and mobile sign-up API, and wired Host event-management buttons for approving pending slots and unconfirming confirmed slots.</x:v>
+      </x:c>
+      <x:c r="G46" s="24" t="str">
+        <x:v>User reported frequent logout friction and asked to proceed without step-by-step confirmations. The app needed durable auto-login behavior plus the next Host management actions.</x:v>
+      </x:c>
+      <x:c r="H46" s="24" t="str">
+        <x:v>mobile/App.tsx; src/lib/mobile/auth.ts; src/app/api/mobile/auth/sign-up/route.ts; src/app/api/mobile/reservations/review/route.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I46" s="24" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-auth-review-export` passed.</x:v>
+      </x:c>
+      <x:c r="J46" s="24" t="str">
+        <x:v>Mobile sign-up follows Supabase email confirmation settings. Host review API permits OUTSIDE_AVAILABLE like the current web approval policy, but blocks explicit host BLOCKED time and confirmed/buffer conflicts.</x:v>
+      </x:c>
+      <x:c r="K46" s="24" t="str">
         <x:v>working tree</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R378a596785ff4164"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb17af5288ad84ca9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2131,7 +2166,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10a7f3f85e184636"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb948909121634664"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2251,7 +2286,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b9b9609dcc844cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8aa18881929a4228"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add mobile event management calendar
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R3b99ca6561cb4339"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R8512d83dfe094a4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rd15b8e613db04780"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R2b5055cc5ec24e7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R70d2858171b54c41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R2bee8eb0bf8142a6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K46" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="WorklogTable" displayName="WorklogTable" ref="A1:K47" headerRowCount="1">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Work_ID"/>
     <x:tableColumn id="2" name="Date_KST"/>
@@ -1980,44 +1980,79 @@
       </x:c>
     </x:row>
     <x:row r="46" ht="84" hidden="0" customHeight="1">
-      <x:c r="A46" s="22" t="str">
+      <x:c r="A46" s="19" t="str">
         <x:v>GPT-20260626-045</x:v>
       </x:c>
-      <x:c r="B46" s="23" t="str">
+      <x:c r="B46" s="20" t="str">
         <x:v>2026-06-26</x:v>
       </x:c>
-      <x:c r="C46" s="24" t="str">
-        <x:v>Codex-GPT-5</x:v>
-      </x:c>
-      <x:c r="D46" s="24" t="str">
+      <x:c r="C46" s="21" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D46" s="21" t="str">
         <x:v>Mobile auth resilience and review actions</x:v>
       </x:c>
-      <x:c r="E46" s="24" t="str">
-        <x:v>Uncommitted</x:v>
-      </x:c>
-      <x:c r="F46" s="24" t="str">
+      <x:c r="E46" s="21" t="str">
+        <x:v>Uncommitted</x:v>
+      </x:c>
+      <x:c r="F46" s="21" t="str">
         <x:v>Hardened native mobile session persistence so dashboard refresh failures no longer clear saved sessions unless the API returns 401, added automatic refresh-token retry for dashboard loads, event creation, code lookup, and review actions, added native email/password sign-up UI and mobile sign-up API, and wired Host event-management buttons for approving pending slots and unconfirming confirmed slots.</x:v>
       </x:c>
-      <x:c r="G46" s="24" t="str">
+      <x:c r="G46" s="21" t="str">
         <x:v>User reported frequent logout friction and asked to proceed without step-by-step confirmations. The app needed durable auto-login behavior plus the next Host management actions.</x:v>
       </x:c>
-      <x:c r="H46" s="24" t="str">
+      <x:c r="H46" s="21" t="str">
         <x:v>mobile/App.tsx; src/lib/mobile/auth.ts; src/app/api/mobile/auth/sign-up/route.ts; src/app/api/mobile/reservations/review/route.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
       </x:c>
-      <x:c r="I46" s="24" t="str">
+      <x:c r="I46" s="21" t="str">
         <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-auth-review-export` passed.</x:v>
       </x:c>
-      <x:c r="J46" s="24" t="str">
+      <x:c r="J46" s="21" t="str">
         <x:v>Mobile sign-up follows Supabase email confirmation settings. Host review API permits OUTSIDE_AVAILABLE like the current web approval policy, but blocks explicit host BLOCKED time and confirmed/buffer conflicts.</x:v>
       </x:c>
-      <x:c r="K46" s="24" t="str">
-        <x:v>working tree</x:v>
+      <x:c r="K46" s="21" t="str">
+        <x:v>working tree</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="108" hidden="0" customHeight="1">
+      <x:c r="A47" s="22" t="str">
+        <x:v>GPT-20260626-046</x:v>
+      </x:c>
+      <x:c r="B47" s="23" t="str">
+        <x:v>2026-06-26</x:v>
+      </x:c>
+      <x:c r="C47" s="24" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D47" s="24" t="str">
+        <x:v>Mobile event management calendar</x:v>
+      </x:c>
+      <x:c r="E47" s="24" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F47" s="24" t="str">
+        <x:v>Added a native read-only Host event-management calendar above the mobile management lists. The calendar has horizontally selectable event dates, a vertical time grid based on event daily hours, compact AM/PM hour labels, half-hour guide lines, and overlaid confirmed/pending candidate blocks with participant names, candidate priority, and time range. Added helpers for confirmed display end times, per-day slot overlap clipping, timeline bounds expansion, clock parsing, and compact date/weekday labels.</x:v>
+      </x:c>
+      <x:c r="G47" s="24" t="str">
+        <x:v>User asked whether the mobile event management page had a calendar. The list-based management page needed a visual schedule surface before deeper mobile editing work.</x:v>
+      </x:c>
+      <x:c r="H47" s="24" t="str">
+        <x:v>mobile/App.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I47" s="24" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, `git diff --check`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-event-calendar-export` passed.</x:v>
+      </x:c>
+      <x:c r="J47" s="24" t="str">
+        <x:v>This calendar is currently read-only. Next mobile management work should add native availability editing, confirmed-slot resizing/buffer editing, and guest reservation editing with the same domain rules as web.</x:v>
+      </x:c>
+      <x:c r="K47" s="24" t="str">
+        <x:v>this commit</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb17af5288ad84ca9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83dc7329e1cc4a61"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2166,7 +2201,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb948909121634664"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7df6bbd1043b42d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2216,7 +2251,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>e0077eb Refine calendar buffer interactions</x:v>
+        <x:v>3fd2cfb Improve mobile auth persistence and review actions</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2224,7 +2259,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>e0077eb Refine calendar buffer interactions</x:v>
+        <x:v>3fd2cfb Improve mobile auth persistence and review actions</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2267,12 +2302,12 @@
         <x:v>npm run typecheck; npm run lint; npm test; npm run build</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="192" hidden="0" customHeight="1">
+    <x:row r="12" ht="36" hidden="0" customHeight="1">
       <x:c r="A12" s="21" t="str">
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Uncommitted: event creation visible-range-only availability selection with no required initial availability, shared 30-minute AM/PM time input, new-event and date-edit label-as-month-picker behavior, date modal daily time editing/wider modal with nested ESC behavior, Host drag preview intent labels/split availability preview with optimistic save to avoid release flicker, taller time calendars, no-inner-scroll widened calendars with mobile day paging, simplified home role-toggle dashboard with Host/Guest tabs, unified event/reservation code entry and resolver, cross-table access-code collision trigger migration, compact home month calendar with label-as-picker, reusable month jump modal for small calendars, weekend color semantics across calendars, 6/11 (목) date headers, full-height in-grid time-calendar week arrows, Host title share/date-edit actions, Host mini week navigator, compact collapsible Host group cards with candidate priority and approval-hover candidate muting, translucent hover-directed buffer-add preview blocks with spinners, custom buffers following confirmed-slot resize, Host approval no longer blocked by outside AVAILABLE ranges, collapsible drag-handle Guest priority lists, larger home calendar previews with group names/status tags on one line, 내 예약 confirmed dated schedules by event name without management codes, event codes beside Host event titles, 30-minute readable calendar grid, Sunday-Saturday event paging, monthly home calendar, confirmed-slot display overrides, public Guest availability splitting around confirmed/buffer ranges, numbered candidate labels, reservation-holder 확정 display blocks plus separate adjusted candidate overlays, additive multi-confirm approval, slot priority_order, Guest priority/reorder/resizing, approved-reservation pending candidate editing with locked confirmed candidates, Host pending overlays above confirmed slots, Host buffer/popover usability fixes, and removal of visible Host rejection controls.</x:v>
+        <x:v>Mobile native app now has auth persistence, sign-up/sign-in, dashboard loading, event creation, code lookup previews, Host event management entry, approve/unconfirm actions, and a read-only management calendar with confirmed/pending blocks. Web app remains the fuller interaction reference for availability editing, buffer editing, and guest reservation editing.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -2280,13 +2315,13 @@
         <x:v>Recommended next work</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Commit/push this UX batch after review, run npx supabase db push for the new access-code trigger migration, smoke-test Host/Guest flows against real Supabase data, then configure Vercel/Supabase deploy URLs.</x:v>
+        <x:v>Continue mobile feature parity: add native Host availability editing, buffer add/remove/resize, confirmed-slot resize/move, reservation candidate editing, guest event booking flow, and deep-link/QR handling after the mobile core screens are functional.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8aa18881929a4228"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcefffca0b74c4a6b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add mobile host availability editing
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R2b5055cc5ec24e7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R70d2858171b54c41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R2bee8eb0bf8142a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Rdf56901b776e4fe8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R3acb1d141dc747c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R73cd6a41357a46a6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -239,9 +239,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -2049,10 +2049,45 @@
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>GPT-20260701-047</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>Mobile availability editing</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F48" t="str">
+        <x:v>Added Supabase-backed mobile Host availability editing. Mobile dashboard payloads now include hosted event time_blocks, a new Bearer-token mobile API route replaces an event's time blocks after verifying Host ownership, and the native event management calendar shows available ranges plus a 30-minute tap-to-toggle edit mode with saving spinner and token refresh retry.</x:v>
+      </x:c>
+      <x:c r="G48" t="str">
+        <x:v>After adding a mobile management calendar, the next missing management capability was changing Host available time from the native app instead of relying on the web UI.</x:v>
+      </x:c>
+      <x:c r="H48" t="str">
+        <x:v>mobile/App.tsx; src/lib/mobile/dashboard.ts; src/app/api/mobile/events/time-blocks/route.ts; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I48" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, `git diff --check`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-timeblocks-export` passed.</x:v>
+      </x:c>
+      <x:c r="J48" t="str">
+        <x:v>Mobile availability editing is immediate-save tap toggling, not drag yet. The endpoint preserves BLOCKED blocks if present, but mobile UI only creates/removes AVAILABLE blocks because personal blocked schedules are planned for a separate personal calendar model.</x:v>
+      </x:c>
+      <x:c r="K48" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83dc7329e1cc4a61"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R020eec448b8d4bd0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2201,7 +2236,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7df6bbd1043b42d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57942cc76a264f5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2251,7 +2286,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>3fd2cfb Improve mobile auth persistence and review actions</x:v>
+        <x:v>8e5adb4 Add mobile event management calendar</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2259,7 +2294,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>3fd2cfb Improve mobile auth persistence and review actions</x:v>
+        <x:v>8e5adb4 Add mobile event management calendar</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2307,7 +2342,7 @@
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Mobile native app now has auth persistence, sign-up/sign-in, dashboard loading, event creation, code lookup previews, Host event management entry, approve/unconfirm actions, and a read-only management calendar with confirmed/pending blocks. Web app remains the fuller interaction reference for availability editing, buffer editing, and guest reservation editing.</x:v>
+        <x:v>Mobile native Host management now includes Supabase-backed availability editing: dashboard time_blocks, mobile save route, 30-minute tap-to-toggle available cells, visible availability overlays, and auth refresh retry.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -2315,13 +2350,13 @@
         <x:v>Recommended next work</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Continue mobile feature parity: add native Host availability editing, buffer add/remove/resize, confirmed-slot resize/move, reservation candidate editing, guest event booking flow, and deep-link/QR handling after the mobile core screens are functional.</x:v>
+        <x:v>Continue mobile feature parity: guest event booking flow, reservation candidate editing, confirmed-slot resize/move, buffer add/remove/resize, QR/deep-link handling, and drag gestures for availability selection.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcefffca0b74c4a6b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9231079354f34cb3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add mobile guest reservation flow
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Rdf56901b776e4fe8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R3acb1d141dc747c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R73cd6a41357a46a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Reb94d1ec9e4e41f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="Rcfe253ad6a27424c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R68eb64cc5d934779"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2084,10 +2084,45 @@
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>GPT-20260701-048</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>Mobile guest reservation flow</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F49" t="str">
+        <x:v>Added a native mobile Guest event reservation screen reached from event-code lookup. The screen loads event detail, shows active-date chips and a 30-minute candidate timeline with availability, confirmed, and buffer overlays, collects headcount/participant names/optional password, creates reservations through the mobile API, and displays the reservation management code. Reworked the mobile reservation creation API so Bearer-token users are recorded as creator/participant instead of falling back to cookie-only web auth. Updated README, mobile README, and TODO to reflect the current native/mobile API state.</x:v>
+      </x:c>
+      <x:c r="G49" t="str">
+        <x:v>The next product gap after Host mobile management was closing the Guest loop so a user can enter an event code and actually submit reservation candidates from the app.</x:v>
+      </x:c>
+      <x:c r="H49" t="str">
+        <x:v>mobile/App.tsx; src/app/api/mobile/reservations/route.ts; README.md; mobile/README.md; TODO.md; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I49" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, `git diff --check`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-reservation-export` passed.</x:v>
+      </x:c>
+      <x:c r="J49" t="str">
+        <x:v>Mobile Guest reservation creation is tap-based for now. Remaining work: native reservation-code management, candidate drag selection/reordering, and Host buffer/confirmed-slot editing parity.</x:v>
+      </x:c>
+      <x:c r="K49" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R020eec448b8d4bd0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c21ed4075e14d2c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2236,7 +2271,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57942cc76a264f5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd630efffbfd4a09"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2286,7 +2321,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>8e5adb4 Add mobile event management calendar</x:v>
+        <x:v>3728046 Add mobile host availability editing</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2294,7 +2329,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>8e5adb4 Add mobile event management calendar</x:v>
+        <x:v>3728046 Add mobile host availability editing</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2342,7 +2377,7 @@
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Mobile native Host management now includes Supabase-backed availability editing: dashboard time_blocks, mobile save route, 30-minute tap-to-toggle available cells, visible availability overlays, and auth refresh retry.</x:v>
+        <x:v>Mobile native Guest flow now includes event-code-to-reservation creation: event detail loading, 30-minute candidate selection, participant/headcount/password entry, mobile reservation API creator linkage, and management code display. Docs were updated to match the current native/mobile API implementation.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -2350,13 +2385,13 @@
         <x:v>Recommended next work</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Continue mobile feature parity: guest event booking flow, reservation candidate editing, confirmed-slot resize/move, buffer add/remove/resize, QR/deep-link handling, and drag gestures for availability selection.</x:v>
+        <x:v>Continue mobile feature parity: reservation-code management/edit/cancel screen, candidate drag selection and priority reordering, Host confirmed-slot resize/move, Host buffer add/remove/resize, and QR/deep-link handling.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9231079354f34cb3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9bb3f8c977e41ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add mobile reservation management
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Reb94d1ec9e4e41f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="Rcfe253ad6a27424c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R68eb64cc5d934779"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Rfb68bcc3f37a43cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R356c7380460540a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rde721fb9c5b14f2c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2119,10 +2119,45 @@
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>GPT-20260701-049</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>Mobile reservation management</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F50" t="str">
+        <x:v>Added a native mobile reservation-code management screen reachable from code lookup and from the joined-reservations list. The screen loads reservation details, shows confirmed slots, edits headcount/participants/password-protected candidate slots, saves through a Bearer-token-aware mobile PUT API, and cancels through a mobile DELETE API. Rebuilt the mobile reservation access-code API around GET/PUT/DELETE management views with creator-aware password bypass, confirmed-slot preservation, participant replacement, pending candidate replacement, cancellation, and dashboard revalidation. Updated README, mobile README, and TODO to reflect the mobile management coverage.</x:v>
+      </x:c>
+      <x:c r="G50" t="str">
+        <x:v>After mobile Guest reservation creation, the next missing app flow was letting users reopen a reservation code to manage or cancel their candidates from mobile.</x:v>
+      </x:c>
+      <x:c r="H50" t="str">
+        <x:v>mobile/App.tsx; src/app/api/mobile/reservations/[accessCode]/route.ts; README.md; mobile/README.md; TODO.md; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I50" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, `git diff --check`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-reservation-manage-export` passed.</x:v>
+      </x:c>
+      <x:c r="J50" t="str">
+        <x:v>Mobile reservation management is tap-based for now. Remaining work: candidate drag selection/reordering, Host confirmed-slot resize/move and buffer editing parity, QR/deep-link handling, and focused mobile API tests.</x:v>
+      </x:c>
+      <x:c r="K50" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c21ed4075e14d2c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R512165c5a1664fcc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2271,7 +2306,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd630efffbfd4a09"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R111fff6da20941af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2321,7 +2356,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>3728046 Add mobile host availability editing</x:v>
+        <x:v>fee9c3d Add mobile guest reservation flow</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2329,7 +2364,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>3728046 Add mobile host availability editing</x:v>
+        <x:v>fee9c3d Add mobile guest reservation flow</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2377,7 +2412,7 @@
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Mobile native Guest flow now includes event-code-to-reservation creation: event detail loading, 30-minute candidate selection, participant/headcount/password entry, mobile reservation API creator linkage, and management code display. Docs were updated to match the current native/mobile API implementation.</x:v>
+        <x:v>Mobile native Guest flow now includes reservation-code management: access-code detail loading, confirmed-slot display, participant/headcount/candidate editing, creator-aware password bypass, cancellation, and updated mobile docs.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -2385,13 +2420,13 @@
         <x:v>Recommended next work</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Continue mobile feature parity: reservation-code management/edit/cancel screen, candidate drag selection and priority reordering, Host confirmed-slot resize/move, Host buffer add/remove/resize, and QR/deep-link handling.</x:v>
+        <x:v>Continue mobile feature parity: candidate drag selection and priority reordering, Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile API route tests.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra9bb3f8c977e41ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b065922b2d54c9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add mobile drag editing
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Rfb68bcc3f37a43cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R356c7380460540a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rde721fb9c5b14f2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R8eafac89b2de4c11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R348cf44f02e14d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R8677d0f4e3b141ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2154,10 +2154,45 @@
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>GPT-20260701-050</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>Mobile drag editing and calendar navigation</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F51" t="str">
+        <x:v>Reworked mobile time editing from one-cell tap actions to drag selection. Host availability editing now opens a local draft mode, updates availability blocks locally while dragging, and sends one time-block save request only when the user taps Save. Guest reservation creation and reservation-code management now use the same 30-minute drag selection layer for adding/removing candidate slots while still posting/putting only on the final submit/save action. Added reusable mobile date navigation with previous/next controls, Today actions, and a year/month picker modal for the home calendar and event time calendars. Updated README, mobile README, and TODO to reflect drag editing and calendar navigation.</x:v>
+      </x:c>
+      <x:c r="G51" t="str">
+        <x:v>The tap-per-cell mobile UX was slow and noisy because Host availability sent a request after each cell change and Guest candidate selection was tedious. Draft-save drag editing makes the app feel closer to the web calendar model while reducing API calls.</x:v>
+      </x:c>
+      <x:c r="H51" t="str">
+        <x:v>mobile/App.tsx; README.md; mobile/README.md; TODO.md; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I51" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, `git diff --check`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-drag-save-export` passed.</x:v>
+      </x:c>
+      <x:c r="J51" t="str">
+        <x:v>Mobile Host availability and Guest candidate selection are now drag-based with batch save/submit. Remaining work: drag-based priority reordering, Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile gesture/API tests.</x:v>
+      </x:c>
+      <x:c r="K51" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R512165c5a1664fcc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ab97361163a4c99"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2306,7 +2341,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R111fff6da20941af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8505c80920544bd0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2356,7 +2391,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>fee9c3d Add mobile guest reservation flow</x:v>
+        <x:v>a4a7d83 Add mobile reservation management</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2364,7 +2399,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>fee9c3d Add mobile guest reservation flow</x:v>
+        <x:v>a4a7d83 Add mobile reservation management</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2412,7 +2447,7 @@
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Mobile native Guest flow now includes reservation-code management: access-code detail loading, confirmed-slot display, participant/headcount/candidate editing, creator-aware password bypass, cancellation, and updated mobile docs.</x:v>
+        <x:v>Mobile time calendars now support drag selection and batch persistence: Host availability edits are local drafts until Save, Guest reservation creation and reservation management candidates are drag-selected until submit/save, and mobile calendars have previous/next, Today, and year/month picker navigation.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -2420,13 +2455,13 @@
         <x:v>Recommended next work</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Continue mobile feature parity: candidate drag selection and priority reordering, Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile API route tests.</x:v>
+        <x:v>Continue mobile feature parity: drag-based priority reordering, Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile gesture/API route tests.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b065922b2d54c9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3452d73c25fd4af3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add mobile calendar drill-down
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R8eafac89b2de4c11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R348cf44f02e14d6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R8677d0f4e3b141ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Ra531756ccf284726"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="Rd52b2ae7417b40fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rb903e5d6c3304a92"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2189,10 +2189,45 @@
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>GPT-20260701-051</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>Mobile calendar drill-down and priority ordering</x:v>
+      </x:c>
+      <x:c r="E52" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F52" t="str">
+        <x:v>Fixed mobile calendar schedule cards so users can drill into the correct detail screen: Host calendar items now open Host event management and Guest reservation items now open reservation management by carrying target metadata through ScheduleItem, MonthCard previews, and upcoming schedule cards. Added drag-based candidate priority reordering for Guest reservation creation and reservation management; candidate order is preserved locally, can be reordered from the candidate list, and is sent to the mobile reservation APIs as the priority order. Updated README, mobile README, and TODO to reflect calendar drill-down and completed priority ordering.</x:v>
+      </x:c>
+      <x:c r="G52" t="str">
+        <x:v>Calendar items were display-only, so tapping a date could show schedules but could not navigate to the relevant event or reservation. Candidate ordering was also still implicit, leaving the next mobile UX gap after drag selection.</x:v>
+      </x:c>
+      <x:c r="H52" t="str">
+        <x:v>mobile/App.tsx; README.md; mobile/README.md; TODO.md; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I52" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, root `npm run typecheck`, `npm run lint`, `npm test`, `npm run build`, `git diff --check`, and `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-calendar-drilldown-export` passed.</x:v>
+      </x:c>
+      <x:c r="J52" t="str">
+        <x:v>Mobile calendar items now navigate to the right detail screens and Guest candidate priorities can be reordered before save/submit. Remaining work: Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile gesture/API tests.</x:v>
+      </x:c>
+      <x:c r="K52" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ab97361163a4c99"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62af80a407c14116"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2341,7 +2376,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8505c80920544bd0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R163a3dd1e66f47d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2391,7 +2426,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>a4a7d83 Add mobile reservation management</x:v>
+        <x:v>de4105a Add mobile drag editing</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2399,7 +2434,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>a4a7d83 Add mobile reservation management</x:v>
+        <x:v>de4105a Add mobile drag editing</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2447,7 +2482,7 @@
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Mobile time calendars now support drag selection and batch persistence: Host availability edits are local drafts until Save, Guest reservation creation and reservation management candidates are drag-selected until submit/save, and mobile calendars have previous/next, Today, and year/month picker navigation.</x:v>
+        <x:v>Mobile calendar schedule items now open Host event management or reservation management, and Guest candidate lists support drag-based priority reordering while preserving that order for create/update API requests.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -2455,13 +2490,13 @@
         <x:v>Recommended next work</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Continue mobile feature parity: drag-based priority reordering, Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile gesture/API route tests.</x:v>
+        <x:v>Continue mobile feature parity: Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile gesture/API route tests.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3452d73c25fd4af3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67d5645b6ba64a5a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add event deletion and mobile save UX
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Ra531756ccf284726"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="Rd52b2ae7417b40fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rb903e5d6c3304a92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R8b8d624067f844ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R0684832e32f3489d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rbfa7a595354b421c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2224,10 +2224,45 @@
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>GPT-20260701-052</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>Event deletion and mobile save/navigation UX</x:v>
+      </x:c>
+      <x:c r="E53" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F53" t="str">
+        <x:v>Added Host event deletion on web and mobile with shared cascading cleanup for reservations, participants, slots, time blocks, active dates, and buffer overrides. Normalized reservation slot priorities after review/update flows and changed Host candidate labels to display list-order numbering. Improved mobile code entry so opening a code immediately routes to Host management, Guest reservation, or reservation management. Added mobile event creation calendar range selection synced with date inputs and removed the confusing static time preview box. Added unsaved-change leave confirmation for draft-save screens, hid the floating plus button while creating, fixed joined tab activation on reservation management, changed reservation management save copy to reservation update, added a web handoff button for event date/default-time edits, and updated project docs.</x:v>
+      </x:c>
+      <x:c r="G53" t="str">
+        <x:v>User reported candidate numbering corruption after unconfirm, missing event deletion, confusing mobile event creation date/time UI, unnecessary code preview, missing save-loss warning, and incorrect joined-tab highlighting.</x:v>
+      </x:c>
+      <x:c r="H53" t="str">
+        <x:v>mobile/App.tsx; src/app/actions/events.ts; src/app/actions/reservations.ts; src/app/api/mobile/events/[eventCode]/route.ts; src/app/api/mobile/reservations/[accessCode]/route.ts; src/app/api/mobile/reservations/review/route.ts; src/app/host/events/[eventId]/page.tsx; src/components/host/event-delete-button.tsx; src/components/host/host-dashboard-shell.tsx; src/lib/events/delete-event.ts; src/lib/reservations/priority.ts; README.md; mobile/README.md; TODO.md; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I53" t="str">
+        <x:v>`npm run typecheck`, `cd mobile &amp;&amp; npx tsc --noEmit`, `npm run lint`, `npm test`, `npm run build`, `git diff --check`, and mobile Expo export passed.</x:v>
+      </x:c>
+      <x:c r="J53" t="str">
+        <x:v>Web/mobile can delete Host events, mobile code entry jumps directly to the right screen, create-date selection supports calendar range selection plus numeric inputs, and draft-save screens warn before discarding unsaved edits. Remaining work: native mobile date/default-time edit parity, Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile API/gesture tests.</x:v>
+      </x:c>
+      <x:c r="K53" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62af80a407c14116"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R876cfff73c2a44ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2376,7 +2411,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R163a3dd1e66f47d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cc9f2265fcc49a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2426,7 +2461,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>de4105a Add mobile drag editing</x:v>
+        <x:v>ed147d4 Add mobile calendar drill-down</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2434,7 +2469,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>de4105a Add mobile drag editing</x:v>
+        <x:v>ed147d4 Add mobile calendar drill-down</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2482,7 +2517,7 @@
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Mobile calendar schedule items now open Host event management or reservation management, and Guest candidate lists support drag-based priority reordering while preserving that order for create/update API requests.</x:v>
+        <x:v>Web/mobile Host event deletion, mobile event creation date picker, immediate code navigation, candidate priority normalization, unsaved-change warnings, and reservation management copy/tab fixes.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -2490,13 +2525,13 @@
         <x:v>Recommended next work</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Continue mobile feature parity: Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile gesture/API route tests.</x:v>
+        <x:v>Continue mobile feature parity: native event date/default-time edit, Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile gesture/API route tests.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67d5645b6ba64a5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d6654da970b41ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add native mobile event settings
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R8b8d624067f844ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R0684832e32f3489d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rbfa7a595354b421c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Rd07aead0a88841f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R261df547f7da46eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rdada61903c5c4a09"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2259,10 +2259,45 @@
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>GPT-20260701-053</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D54" t="str">
+        <x:v>Mobile event settings and access routing</x:v>
+      </x:c>
+      <x:c r="E54" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F54" t="str">
+        <x:v>Replaced the mobile Host event management web handoff for date/default-time changes with an in-app edit modal that reuses the synced calendar range picker, date inputs, and daily time inputs. Added a PATCH mobile event route with Host token validation to save active dates, date bounds, and default daily time bounds. Updated mobile event-code resolution so if a logged-in non-Host user already has a PENDING or APPROVED reservation for that event as creator or participant, entering the event code opens reservation management instead of the new reservation screen. Updated README/TODO mobile coverage notes.</x:v>
+      </x:c>
+      <x:c r="G54" t="str">
+        <x:v>User wanted date/default-time edits to stay inside the app, and pointed out that event-code lookup should resume an existing reservation rather than creating a duplicate reservation flow.</x:v>
+      </x:c>
+      <x:c r="H54" t="str">
+        <x:v>mobile/App.tsx; src/app/api/mobile/events/[eventCode]/route.ts; src/app/api/mobile/access/resolve/route.ts; README.md; mobile/README.md; TODO.md; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I54" t="str">
+        <x:v>`npm run typecheck`, `cd mobile &amp;&amp; npx tsc --noEmit`, and `npm run lint` passed before log update; full verification pending this commit.</x:v>
+      </x:c>
+      <x:c r="J54" t="str">
+        <x:v>Mobile Host event settings can now be edited natively, and mobile event-code lookup resumes existing pending/approved reservations for the logged-in user. Remaining work: Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile API/gesture tests.</x:v>
+      </x:c>
+      <x:c r="K54" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R876cfff73c2a44ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac318700851c4793"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2411,7 +2446,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7cc9f2265fcc49a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R879a6fe858c147e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2461,7 +2496,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>ed147d4 Add mobile calendar drill-down</x:v>
+        <x:v>213aa19 Add event deletion and mobile save UX</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2469,7 +2504,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>ed147d4 Add mobile calendar drill-down</x:v>
+        <x:v>213aa19 Add event deletion and mobile save UX</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2517,7 +2552,7 @@
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Web/mobile Host event deletion, mobile event creation date picker, immediate code navigation, candidate priority normalization, unsaved-change warnings, and reservation management copy/tab fixes.</x:v>
+        <x:v>Mobile Host event date/default-time edits are native, and mobile event-code lookup opens existing pending/approved reservations for the logged-in user.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -2525,13 +2560,13 @@
         <x:v>Recommended next work</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Continue mobile feature parity: native event date/default-time edit, Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile gesture/API route tests.</x:v>
+        <x:v>Continue mobile feature parity: Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile gesture/API route tests.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d6654da970b41ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbad06a7633c04d2a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add mobile active date toggles
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="Rd07aead0a88841f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R261df547f7da46eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rdada61903c5c4a09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R0e7cc2281c094a62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R31a2df703b7c4351"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R3cea21dfddf04885"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2294,10 +2294,45 @@
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
+        <x:v>GPT-20260701-054</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>Mobile active date toggles and midnight presets</x:v>
+      </x:c>
+      <x:c r="E55" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F55" t="str">
+        <x:v>Updated the native mobile active-date picker used by event creation and Host date/default-time editing so dates can be toggled individually by tap or changed in batches by drag. Synced numeric date inputs with the active date list and preserved discontinuous active dates in mobile Host dashboard data. Added 0시 and 자정 preset check controls beside the default start/end time labels in both mobile event creation and mobile Host event date/default-time editing. Updated README/TODO mobile coverage notes.</x:v>
+      </x:c>
+      <x:c r="G55" t="str">
+        <x:v>User wanted mobile date selection to support direct individual activation/deactivation instead of only drag range behavior, and asked for the same 0시/자정 shortcut controls on mobile.</x:v>
+      </x:c>
+      <x:c r="H55" t="str">
+        <x:v>mobile/App.tsx; src/lib/mobile/dashboard.ts; README.md; mobile/README.md; TODO.md; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I55" t="str">
+        <x:v>`npm run typecheck`, `cd mobile &amp;&amp; npx tsc --noEmit`, `npm run lint`, `npm test`, `npm run build`, `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-active-dates-export`, and `git diff --check` passed.</x:v>
+      </x:c>
+      <x:c r="J55" t="str">
+        <x:v>Mobile event creation and Host event date/default-time editing now support tap/drag active-date toggles plus 0시/자정 presets. Remaining work: Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile API/gesture tests.</x:v>
+      </x:c>
+      <x:c r="K55" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac318700851c4793"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34657d999f01406c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2446,7 +2481,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R879a6fe858c147e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b0cc086fd2940ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2496,7 +2531,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>213aa19 Add event deletion and mobile save UX</x:v>
+        <x:v>d17f9c4 Add native mobile event settings</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2504,7 +2539,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>213aa19 Add event deletion and mobile save UX</x:v>
+        <x:v>d17f9c4 Add native mobile event settings</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2552,7 +2587,7 @@
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Mobile Host event date/default-time edits are native, and mobile event-code lookup opens existing pending/approved reservations for the logged-in user.</x:v>
+        <x:v>Mobile event creation and Host event date/default-time editing support tap/drag active-date toggles and 0시/자정 time presets.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -2566,7 +2601,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbad06a7633c04d2a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4c759260f2a4a2e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix mobile calendar navigation
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R0e7cc2281c094a62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R31a2df703b7c4351"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R3cea21dfddf04885"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R96f3d8d69d6b488d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R6f85194061df41f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R706aef3bfcc541aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2329,10 +2329,45 @@
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="str">
+        <x:v>GPT-20260701-055</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D56" t="str">
+        <x:v>Mobile calendar navigation and schedule filters</x:v>
+      </x:c>
+      <x:c r="E56" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F56" t="str">
+        <x:v>Fixed mobile active-date deactivation so the UI can temporarily hold zero selected dates and only validates one-or-more active dates on save/create. Updated mobile event create and Host date/default-time update API normalization so an explicit empty activeDates array is rejected instead of silently restoring the full date range. Added source-aware detail navigation so opening an event/reservation from the calendar returns to the calendar on back, while openings from 내 이벤트 or 참여 return to their source tabs. Split the mobile calendar schedule list into upcoming and past toggles, sorted by proximity to today, and excluded Host pending slots from the upcoming/past list while keeping their month markers and date previews. Updated README/TODO mobile notes.</x:v>
+      </x:c>
+      <x:c r="G56" t="str">
+        <x:v>User reported date deactivation was not working, wanted the same create/edit active-date logic, and clarified calendar detail back behavior plus upcoming/past schedule filtering.</x:v>
+      </x:c>
+      <x:c r="H56" t="str">
+        <x:v>mobile/App.tsx; src/app/api/mobile/events/route.ts; src/app/api/mobile/events/[eventCode]/route.ts; README.md; mobile/README.md; TODO.md; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I56" t="str">
+        <x:v>`npm run typecheck`, `cd mobile &amp;&amp; npx tsc --noEmit`, `npm run lint`, `npm test`, `npm run build`, `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-calendar-nav-export`, and `git diff --check` passed.</x:v>
+      </x:c>
+      <x:c r="J56" t="str">
+        <x:v>Mobile active-date deactivation is consistent across event creation and editing, calendar detail back navigation now respects the source tab, and the calendar schedule list separates upcoming/past items while keeping Host pending items as markers only. Remaining work: Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile gesture/API route tests.</x:v>
+      </x:c>
+      <x:c r="K56" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34657d999f01406c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28c34dcb52a5461c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2481,7 +2516,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b0cc086fd2940ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd572fe2736e4dad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2531,7 +2566,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>d17f9c4 Add native mobile event settings</x:v>
+        <x:v>05de688 Add mobile active date toggles</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2539,7 +2574,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>d17f9c4 Add native mobile event settings</x:v>
+        <x:v>05de688 Add mobile active date toggles</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2587,7 +2622,7 @@
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Mobile event creation and Host event date/default-time editing support tap/drag active-date toggles and 0시/자정 time presets.</x:v>
+        <x:v>Mobile active-date deactivation, source-aware calendar detail back navigation, and upcoming/past calendar schedule filters.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -2601,7 +2636,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4c759260f2a4a2e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb182b2098944704"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Expo Go startup scripts
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R96f3d8d69d6b488d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R6f85194061df41f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R706aef3bfcc541aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R6a8373f467bf473d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R8d3eaa6f4b974af8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R0a097d6d51964201"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2364,10 +2364,45 @@
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="str">
+        <x:v>GPT-20260701-056</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D57" t="str">
+        <x:v>Expo Go local startup scripts</x:v>
+      </x:c>
+      <x:c r="E57" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F57" t="str">
+        <x:v>Changed the mobile Android default script to local/offline localhost Expo Go startup to avoid Expo server manifest lookup failures such as UnexpectedServerData: No returned query result. Added explicit LAN and tunnel scripts for physical-device Expo Go testing, plus start:local/start:lan/start:tunnel helpers. Documented emulator vs physical phone commands and the workaround for stale Metro processes occupying port 8081.</x:v>
+      </x:c>
+      <x:c r="G57" t="str">
+        <x:v>User reported Expo Go failing to open with UnexpectedServerData. Local inspection showed the online android script could hit Expo server query failures and 8081 was already occupied by an existing node/Metro process.</x:v>
+      </x:c>
+      <x:c r="H57" t="str">
+        <x:v>mobile/package.json; mobile/README.md; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I57" t="str">
+        <x:v>`cd mobile &amp;&amp; npm pkg get scripts`, `cd mobile &amp;&amp; npx tsc --noEmit`, `npm run typecheck`, `npm run lint`, and `git diff --check` passed.</x:v>
+      </x:c>
+      <x:c r="J57" t="str">
+        <x:v>Mobile Expo startup now defaults to offline localhost for Android emulator use, with separate LAN/tunnel scripts for physical phone testing. Remaining note: if 8081 is held by an old Metro process, stop it with Ctrl+C or run with --port 8082.</x:v>
+      </x:c>
+      <x:c r="K57" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28c34dcb52a5461c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R996a43a4c2904638"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2516,7 +2551,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd572fe2736e4dad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3945939585cf45cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2566,7 +2601,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>05de688 Add mobile active date toggles</x:v>
+        <x:v>a0ec01a Fix mobile calendar navigation</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2574,7 +2609,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>05de688 Add mobile active date toggles</x:v>
+        <x:v>a0ec01a Fix mobile calendar navigation</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2622,7 +2657,7 @@
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Mobile active-date deactivation, source-aware calendar detail back navigation, and upcoming/past calendar schedule filters.</x:v>
+        <x:v>Mobile Expo Go startup scripts now separate offline emulator use from LAN/tunnel physical-device use.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -2636,7 +2671,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb182b2098944704"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb4ccb593519440f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix mobile gesture selection
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R6a8373f467bf473d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R8d3eaa6f4b974af8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R0a097d6d51964201"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R9fcf1a44e9c446df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R7c2b68f872fe4b68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Red3aef9836ac46ac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2399,10 +2399,45 @@
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
+    <x:row r="58">
+      <x:c r="A58" t="str">
+        <x:v>GPT-20260701-057</x:v>
+      </x:c>
+      <x:c r="B58" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C58" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D58" t="str">
+        <x:v>Mobile gesture selection fixes</x:v>
+      </x:c>
+      <x:c r="E58" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F58" t="str">
+        <x:v>Fixed mobile date selection so event creation and host date editing both support tap toggle, active-to-inactive drag, and inactive-to-active drag with the same rounded preview styling as committed dates. Reworked mobile timeline drag commits for host availability and guest candidate slots so fast taps and drags commit after render without React setState-in-render warnings. Aligned add/remove drag previews to the exact 30-minute grid cell top, height, and horizontal inset.</x:v>
+      </x:c>
+      <x:c r="G58" t="str">
+        <x:v>User reported date tap/deactivation not working, a React warning after dragging availability then tapping a cell to remove it, and host/guest drag preview boxes not snapping visually to the grid.</x:v>
+      </x:c>
+      <x:c r="H58" t="str">
+        <x:v>mobile/App.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I58" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, `npm run lint`, `npm run typecheck`, `npm test`, `npm run build`, `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-gesture-export`, and `git diff --check` passed.</x:v>
+      </x:c>
+      <x:c r="J58" t="str">
+        <x:v>Mobile date selection and timeline drag previews now share consistent commit behavior and grid-aligned visuals. Remaining unrelated local dependency changes in mobile/package.json and mobile/package-lock.json were intentionally left unstaged.</x:v>
+      </x:c>
+      <x:c r="K58" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R996a43a4c2904638"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c73f52f782d4335"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2551,7 +2586,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3945939585cf45cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raef6d370d93144c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2601,7 +2636,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>a0ec01a Fix mobile calendar navigation</x:v>
+        <x:v>56fb868 Fix Expo Go startup scripts</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2609,7 +2644,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>a0ec01a Fix mobile calendar navigation</x:v>
+        <x:v>56fb868 Fix Expo Go startup scripts</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2657,7 +2692,7 @@
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Mobile Expo Go startup scripts now separate offline emulator use from LAN/tunnel physical-device use.</x:v>
+        <x:v>Mobile date picker and timeline drag selection now commit fast taps safely, support active/inactive date drag toggles, and draw grid-aligned previews.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -2665,13 +2700,13 @@
         <x:v>Recommended next work</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Continue mobile feature parity: Host confirmed-slot resize/move, Host buffer add/remove/resize, QR/deep-link handling, and focused mobile gesture/API route tests.</x:v>
+        <x:v>Continue mobile feature parity: Host confirmed-slot resize/move, Host buffer add/remove/resize, event QR/deep-link handling, and focused mobile gesture/API route tests.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb4ccb593519440f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra87df61401dc4236"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix mobile tap cancellation
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R9fcf1a44e9c446df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R7c2b68f872fe4b68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Red3aef9836ac46ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R268087b50250477f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R25d12736bcf14275"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rc247e9532f9e4942"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2434,10 +2434,45 @@
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
+    <x:row r="59">
+      <x:c r="A59" t="str">
+        <x:v>GPT-20260701-058</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D59" t="str">
+        <x:v>Mobile tap cancellation reliability</x:v>
+      </x:c>
+      <x:c r="E59" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F59" t="str">
+        <x:v>Separated tap cancellation from drag responder handling on mobile. Date cells now use direct Pressable taps for single-day activate/deactivate while PanResponder only takes over after movement for range drags. Timeline cells for host availability and guest candidate slots now have transparent 30-minute Pressable hit targets for one-cell add/remove, with drag still handled by the shared drag layer after movement begins.</x:v>
+      </x:c>
+      <x:c r="G59" t="str">
+        <x:v>User reported cancellation still did not work after the prior gesture fix. The risky path was relying on PanResponder start/release for simple taps, so single-cell cancellation needed a direct press path instead of a drag responder commit.</x:v>
+      </x:c>
+      <x:c r="H59" t="str">
+        <x:v>mobile/App.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I59" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, `npm run lint`, `npm run typecheck`, `npm test`, `npm run build`, `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-cancel-export`, and `git diff --check` passed.</x:v>
+      </x:c>
+      <x:c r="J59" t="str">
+        <x:v>Mobile single-date and single-time-cell cancellation now uses direct tap handlers. Drag gestures still support range changes once movement exceeds the small threshold. Remaining unrelated local dependency changes in mobile/package.json and mobile/package-lock.json were intentionally left unstaged.</x:v>
+      </x:c>
+      <x:c r="K59" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c73f52f782d4335"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c34e99fab294293"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2586,7 +2621,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raef6d370d93144c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R362124790ae44d6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2636,7 +2671,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>56fb868 Fix Expo Go startup scripts</x:v>
+        <x:v>bab9f19 Fix mobile gesture selection</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2644,7 +2679,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>56fb868 Fix Expo Go startup scripts</x:v>
+        <x:v>bab9f19 Fix mobile gesture selection</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2692,7 +2727,7 @@
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Mobile date picker and timeline drag selection now commit fast taps safely, support active/inactive date drag toggles, and draw grid-aligned previews.</x:v>
+        <x:v>Mobile tap cancellation for date cells and 30-minute timeline cells now bypasses PanResponder start/release and uses direct Pressable hit targets.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -2706,7 +2741,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra87df61401dc4236"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75dfc039a8a14968"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix mobile drag coordinate tracking
</commit_message>
<xml_diff>
--- a/handoff/GradPhotoTime_Worklog.xlsx
+++ b/handoff/GradPhotoTime_Worklog.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R268087b50250477f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R25d12736bcf14275"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="Rc247e9532f9e4942"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worklog" sheetId="1" r:id="R2f4c6d53a1ff4b9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handoff Protocol" sheetId="2" r:id="R066a71e63a874f1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current State" sheetId="3" r:id="R42b6b594da8e47a6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2469,10 +2469,45 @@
         <x:v>this commit</x:v>
       </x:c>
     </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="str">
+        <x:v>GPT-20260701-059</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>2026-07-01</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
+        <x:v>Codex-GPT-5</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>Mobile drag coordinate repair</x:v>
+      </x:c>
+      <x:c r="E60" t="str">
+        <x:v>Committed</x:v>
+      </x:c>
+      <x:c r="F60" t="str">
+        <x:v>Repaired mobile drag coordinate handling after adding tap hit targets. Date and timeline drags now record the pressed cell's absolute grid-local start coordinate on press-in and compute current preview/commit positions from gesture dx/dy instead of event location values that can be relative to a child Pressable. Lowered drag recognition threshold from 4px to 1px so range edits begin as soon as the user moves.</x:v>
+      </x:c>
+      <x:c r="G60" t="str">
+        <x:v>User reported drag UX felt stiff and that host availability/guest candidate drags created previews and committed blocks at the wrong top position. The root cause was child Pressable hit targets changing event location coordinates while the shared drag layer still interpreted them as parent-local coordinates.</x:v>
+      </x:c>
+      <x:c r="H60" t="str">
+        <x:v>mobile/App.tsx; handoff/GradPhotoTime_Worklog.xlsx</x:v>
+      </x:c>
+      <x:c r="I60" t="str">
+        <x:v>`cd mobile &amp;&amp; npx tsc --noEmit`, `npm run lint`, `npm run typecheck`, `npm test`, `npm run build`, `cd mobile &amp;&amp; npx expo export --platform android --output-dir /private/tmp/gradphoto-mobile-drag-export`, and `git diff --check` passed.</x:v>
+      </x:c>
+      <x:c r="J60" t="str">
+        <x:v>Mobile date range, host availability, and guest candidate drags now track the user's actual start cell and movement distance, including back-and-forth shrinking/expanding. Remaining unrelated local dependency changes in mobile/package.json and mobile/package-lock.json were intentionally left unstaged.</x:v>
+      </x:c>
+      <x:c r="K60" t="str">
+        <x:v>this commit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c34e99fab294293"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3b66ba528504f8c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2621,7 +2656,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R362124790ae44d6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R754c1a093792432b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2671,7 +2706,7 @@
         <x:v>Pushed commit before current work</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>bab9f19 Fix mobile gesture selection</x:v>
+        <x:v>9d37e07 Fix mobile tap cancellation</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -2679,7 +2714,7 @@
         <x:v>Local commit before current work</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
-        <x:v>bab9f19 Fix mobile gesture selection</x:v>
+        <x:v>9d37e07 Fix mobile tap cancellation</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -2727,7 +2762,7 @@
         <x:v>Current commit scope</x:v>
       </x:c>
       <x:c r="B12" s="21" t="str">
-        <x:v>Mobile tap cancellation for date cells and 30-minute timeline cells now bypasses PanResponder start/release and uses direct Pressable hit targets.</x:v>
+        <x:v>Mobile drag coordinates now use press-in grid-local start coordinates plus gesture dx/dy, preventing child Pressable location offsets from moving previews to the wrong slot.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -2741,7 +2776,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75dfc039a8a14968"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7129770b818c4735"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>